<commit_message>
docs: record Task 7 verification, the live OTP check and the human-timing protocol in the tracker
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/tracking/SELA_Progress_Tracker.xlsx
+++ b/docs/tracking/SELA_Progress_Tracker.xlsx
@@ -14,8 +14,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Tracker'!$A$1:$K$32</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Change Log'!$A$1:$H$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Tracker'!$A$1:$K$34</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Change Log'!$A$1:$H$23</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Traceability'!$A$1:$G$59</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -982,7 +982,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K32"/>
+  <dimension ref="A1:K34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1681,7 +1681,7 @@
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>Pending Verification</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="F13" s="7" t="inlineStr">
@@ -1706,12 +1706,12 @@
       </c>
       <c r="J13" s="7" t="inlineStr">
         <is>
-          <t>Tests so far used in-process Redis (miniredis) and a fake SMTP server; run the stack with docker compose and sign in through Mailpit's inbox once Docker is available</t>
+          <t>Verified live on 2026-09-20 against docker compose Redis 7 (password) and Mailpit with the real cmd/api, via apps/web/tests/e2e/auth-live.spec.ts (6 checks, all pass, no service change needed) and the host happy path (sign-in read from the Mailpit inbox). Checked: email delivery and format, wrong/right code, cookie flags, no token in body, single use, hashes-only in Redis, rate limit (429 + Retry-After), lockout after 5 wrong codes.</t>
         </is>
       </c>
       <c r="K13" s="7" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -2217,147 +2217,179 @@
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>Task 7: Verify milestone outcome — End-to-end test and timed usability check against the 3-minute target</t>
+          <t>Task 7: Verify milestone outcome — Real-stack end-to-end test and automated timing against the 3-minute target (the human timing is T7.2)</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>apps/web (tests/e2e)</t>
+          <t>apps/web (tests/e2e), scripts/e2e.sh, scripts/check.sh</t>
         </is>
       </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F23" s="7" t="inlineStr"/>
-      <c r="G23" s="7" t="inlineStr"/>
-      <c r="H23" s="7" t="inlineStr"/>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F23" s="7" t="inlineStr">
+        <is>
+          <t>56159ff 70c75d0 44e0983</t>
+        </is>
+      </c>
+      <c r="G23" s="7" t="inlineStr">
+        <is>
+          <t>29d31b5 fcdfe29 6037092 96d0a2a 7b11984</t>
+        </is>
+      </c>
+      <c r="H23" s="7" t="inlineStr">
+        <is>
+          <t>n/a for e2e; helper unit tests 17 (168 unit tests total, web coverage 99.7% lines / 90.2% branches); 10 e2e tests pass on the real stack</t>
+        </is>
+      </c>
       <c r="I23" s="7" t="inlineStr">
         <is>
-          <t>FR-01.1, FR-01.2, FR-01.3</t>
+          <t>FR-01.1, FR-01.2, FR-01.3, FR-09.1</t>
         </is>
       </c>
       <c r="J23" s="7" t="inlineStr">
         <is>
-          <t>Playwright happy path; median setup time of 3-5 first-time hosts recorded in the PRD metrics</t>
+          <t>Playwright (installed Chrome) against real cmd/api + Postgres + Redis + Mailpit via scripts/e2e.sh, also run by scripts/check.sh: sign-in from the Mailpit inbox, category, form, event, short link, QR PNG decoded back to the link, PNG/SVG downloads, cookie flags, guest resolver, reload, not-found, signed-out bounce. Scripted setup time 2.7-2.8 s warm (8.5 s cold first run) vs the 180 s target. Tooling commits 58b435f, d34c798.</t>
         </is>
       </c>
       <c r="K23" s="7" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
         <is>
-          <t>Milestone 2: Guest captures and uploads</t>
+          <t>Milestone 1: Host creates an event</t>
         </is>
       </c>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>M2.1</t>
+          <t>T7.2</t>
         </is>
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>Milestone 2 (not yet planned) — Guest scan, camera, upload with quota, gallery upload</t>
+          <t>Task 7: Verify milestone outcome — Human timed usability check: median setup time of 3-5 first-time hosts against the PRD metric (3 minutes or less, no documentation)</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>apps/web, services/media, services/event</t>
+          <t>docs/tracking (usability_sessions.csv)</t>
         </is>
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F24" s="7" t="inlineStr"/>
-      <c r="G24" s="7" t="inlineStr"/>
-      <c r="H24" s="7" t="inlineStr"/>
+          <t>Pending Verification</t>
+        </is>
+      </c>
+      <c r="F24" s="7" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="G24" s="7" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H24" s="7" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
       <c r="I24" s="7" t="inlineStr">
         <is>
-          <t>FR-02.1-02.4, FR-03.1-03.6, FR-04.1-04.2, FR-SEC.2, FR-SEC.3</t>
+          <t>FR-01.1, FR-01.2, FR-01.3</t>
         </is>
       </c>
       <c r="J24" s="7" t="inlineStr">
         <is>
-          <t>Guest session, PWA camera pipeline, Redis shot quota, upload validation</t>
+          <t>Protocol in docs/tracking/README.md and an empty session template docs/tracking/usability_sessions.csv exist; no sessions have been run. Needs 3-5 first-time hosts; the median of total_s is compared with 180 s and recorded in the PRD metrics table. Automation (T7.1) cannot stand in for it.</t>
         </is>
       </c>
       <c r="K24" s="7" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
         <is>
-          <t>Milestone 3: Role-correct gallery</t>
+          <t>Milestone 1: Host creates an event</t>
         </is>
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>M3.1</t>
+          <t>T7.3</t>
         </is>
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>Milestone 3 (not yet planned) — Role-correct gallery, reveal timer, real-time channels</t>
+          <t>Task 7: Verify milestone outcome — Docs sync (FSD v2.9) and tracker update for Task 7</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>services/gallery, services/realtime</t>
+          <t>docs (FSD v2.9), docs/tracking, CLAUDE.md</t>
         </is>
       </c>
       <c r="E25" s="7" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F25" s="7" t="inlineStr"/>
-      <c r="G25" s="7" t="inlineStr"/>
-      <c r="H25" s="7" t="inlineStr"/>
-      <c r="I25" s="7" t="inlineStr">
-        <is>
-          <t>FR-05.1-05.6</t>
-        </is>
-      </c>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F25" s="7" t="inlineStr">
+        <is>
+          <t>n/a (documentation)</t>
+        </is>
+      </c>
+      <c r="G25" s="7" t="inlineStr">
+        <is>
+          <t>n/a (FSD/CLAUDE.md are gitignored .md files; the tracker files are versioned)</t>
+        </is>
+      </c>
+      <c r="H25" s="7" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I25" s="7" t="inlineStr"/>
       <c r="J25" s="7" t="inlineStr">
         <is>
-          <t>Host sees all media, guest only their own, WebSocket channels split by role</t>
+          <t>FSD change row, 8.6 live-verification note, 10.1 e2e/timing note, 11.1; tracking README timed-check protocol; this tracker</t>
         </is>
       </c>
       <c r="K25" s="7" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
         <is>
-          <t>Milestone 4: Moderate and export</t>
+          <t>Milestone 2: Guest captures and uploads</t>
         </is>
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>M4.1</t>
+          <t>M2.1</t>
         </is>
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>Milestone 4 (not yet planned) — Moderation and full-gallery ZIP export</t>
+          <t>Milestone 2 (not yet planned) — Guest scan, camera, upload with quota, gallery upload</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>services/gallery, services/media</t>
+          <t>apps/web, services/media, services/event</t>
         </is>
       </c>
       <c r="E26" s="7" t="inlineStr">
@@ -2370,12 +2402,12 @@
       <c r="H26" s="7" t="inlineStr"/>
       <c r="I26" s="7" t="inlineStr">
         <is>
-          <t>FR-06.1-06.4, FR-07.1-07.3</t>
+          <t>FR-02.1-02.4, FR-03.1-03.6, FR-04.1-04.2, FR-SEC.2, FR-SEC.3</t>
         </is>
       </c>
       <c r="J26" s="7" t="inlineStr">
         <is>
-          <t>Hide/delete, asynchronous ZIP export, share links</t>
+          <t>Guest session, PWA camera pipeline, Redis shot quota, upload validation</t>
         </is>
       </c>
       <c r="K26" s="7" t="inlineStr">
@@ -2387,22 +2419,22 @@
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
         <is>
-          <t>Milestone 5: Plans and payment</t>
+          <t>Milestone 3: Role-correct gallery</t>
         </is>
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>M5.1</t>
+          <t>M3.1</t>
         </is>
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>Milestone 5 (not yet planned) — Plans, package recommendation and payment (QRIS, e-wallet, card)</t>
+          <t>Milestone 3 (not yet planned) — Role-correct gallery, reveal timer, real-time channels</t>
         </is>
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>services/payment, services/event</t>
+          <t>services/gallery, services/realtime</t>
         </is>
       </c>
       <c r="E27" s="7" t="inlineStr">
@@ -2415,12 +2447,12 @@
       <c r="H27" s="7" t="inlineStr"/>
       <c r="I27" s="7" t="inlineStr">
         <is>
-          <t>FR-01.5, FR-01.6, FR-09.2, FR-09.3</t>
+          <t>FR-05.1-05.6</t>
         </is>
       </c>
       <c r="J27" s="7" t="inlineStr">
         <is>
-          <t>Free and paid tiers by event scale; micro-payments; transaction history</t>
+          <t>Host sees all media, guest only their own, WebSocket channels split by role</t>
         </is>
       </c>
       <c r="K27" s="7" t="inlineStr">
@@ -2432,22 +2464,22 @@
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>Milestone 6: Privacy and compliance readiness</t>
+          <t>Milestone 4: Moderate and export</t>
         </is>
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>M6.1</t>
+          <t>M4.1</t>
         </is>
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>Milestone 6 (not yet planned) — Privacy and compliance readiness</t>
+          <t>Milestone 4 (not yet planned) — Moderation and full-gallery ZIP export</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>cross-cutting</t>
+          <t>services/gallery, services/media</t>
         </is>
       </c>
       <c r="E28" s="7" t="inlineStr">
@@ -2460,12 +2492,12 @@
       <c r="H28" s="7" t="inlineStr"/>
       <c r="I28" s="7" t="inlineStr">
         <is>
-          <t>FR-SEC.1, FR-SEC.5-SEC.8, FR-SEC.10</t>
+          <t>FR-06.1-06.4, FR-07.1-07.3</t>
         </is>
       </c>
       <c r="J28" s="7" t="inlineStr">
         <is>
-          <t>PII column encryption with a blind index, audit log, retention and deletion, child-event defaults, noindex headers</t>
+          <t>Hide/delete, asynchronous ZIP export, share links</t>
         </is>
       </c>
       <c r="K28" s="7" t="inlineStr">
@@ -2477,22 +2509,22 @@
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
         <is>
-          <t>Milestone 7: Closed beta</t>
+          <t>Milestone 5: Plans and payment</t>
         </is>
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>M7.1</t>
+          <t>M5.1</t>
         </is>
       </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>Milestone 7 (not yet planned) — Closed beta across wedding, graduation and birthday events</t>
+          <t>Milestone 5 (not yet planned) — Plans, package recommendation and payment (QRIS, e-wallet, card)</t>
         </is>
       </c>
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>operations</t>
+          <t>services/payment, services/event</t>
         </is>
       </c>
       <c r="E29" s="7" t="inlineStr">
@@ -2503,10 +2535,14 @@
       <c r="F29" s="7" t="inlineStr"/>
       <c r="G29" s="7" t="inlineStr"/>
       <c r="H29" s="7" t="inlineStr"/>
-      <c r="I29" s="7" t="inlineStr"/>
+      <c r="I29" s="7" t="inlineStr">
+        <is>
+          <t>FR-01.5, FR-01.6, FR-09.2, FR-09.3</t>
+        </is>
+      </c>
       <c r="J29" s="7" t="inlineStr">
         <is>
-          <t>Validate the hypothesis and fill the TBD success metrics in the PRD</t>
+          <t>Free and paid tiers by event scale; micro-payments; transaction history</t>
         </is>
       </c>
       <c r="K29" s="7" t="inlineStr">
@@ -2518,22 +2554,22 @@
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
         <is>
-          <t>Backlog: Should-have and later phases</t>
+          <t>Milestone 6: Privacy and compliance readiness</t>
         </is>
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>BL.1</t>
+          <t>M6.1</t>
         </is>
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>Backlog: Notifications — Scheduled and transactional email/WhatsApp notifications</t>
+          <t>Milestone 6 (not yet planned) — Privacy and compliance readiness</t>
         </is>
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>services/notification</t>
+          <t>cross-cutting</t>
         </is>
       </c>
       <c r="E30" s="7" t="inlineStr">
@@ -2546,12 +2582,12 @@
       <c r="H30" s="7" t="inlineStr"/>
       <c r="I30" s="7" t="inlineStr">
         <is>
-          <t>FR-08.1-08.2</t>
+          <t>FR-SEC.1, FR-SEC.5-SEC.8, FR-SEC.10</t>
         </is>
       </c>
       <c r="J30" s="7" t="inlineStr">
         <is>
-          <t>Event reminders, reveal notices, expiry warnings</t>
+          <t>PII column encryption with a blind index, audit log, retention and deletion, child-event defaults, noindex headers</t>
         </is>
       </c>
       <c r="K30" s="7" t="inlineStr">
@@ -2563,22 +2599,22 @@
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
         <is>
-          <t>Backlog: Should-have and later phases</t>
+          <t>Milestone 7: Closed beta</t>
         </is>
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>BL.2</t>
+          <t>M7.1</t>
         </is>
       </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
-          <t>Backlog: Hall of Fame — Host-curated highlights visible to guests</t>
+          <t>Milestone 7 (not yet planned) — Closed beta across wedding, graduation and birthday events</t>
         </is>
       </c>
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>services/gallery</t>
+          <t>operations</t>
         </is>
       </c>
       <c r="E31" s="7" t="inlineStr">
@@ -2589,14 +2625,10 @@
       <c r="F31" s="7" t="inlineStr"/>
       <c r="G31" s="7" t="inlineStr"/>
       <c r="H31" s="7" t="inlineStr"/>
-      <c r="I31" s="7" t="inlineStr">
-        <is>
-          <t>FR-11.1-11.5</t>
-        </is>
-      </c>
+      <c r="I31" s="7" t="inlineStr"/>
       <c r="J31" s="7" t="inlineStr">
         <is>
-          <t>Curation, ordering and sharing of the best photos</t>
+          <t>Validate the hypothesis and fill the TBD success metrics in the PRD</t>
         </is>
       </c>
       <c r="K31" s="7" t="inlineStr">
@@ -2613,17 +2645,17 @@
       </c>
       <c r="B32" s="7" t="inlineStr">
         <is>
-          <t>BL.3</t>
+          <t>BL.1</t>
         </is>
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>Backlog: Personal/Instant Mode (v1.1) — Capture without an event and send results to several recipients</t>
+          <t>Backlog: Notifications — Scheduled and transactional email/WhatsApp notifications</t>
         </is>
       </c>
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>apps/web, services/media</t>
+          <t>services/notification</t>
         </is>
       </c>
       <c r="E32" s="7" t="inlineStr">
@@ -2636,23 +2668,113 @@
       <c r="H32" s="7" t="inlineStr"/>
       <c r="I32" s="7" t="inlineStr">
         <is>
+          <t>FR-08.1-08.2</t>
+        </is>
+      </c>
+      <c r="J32" s="7" t="inlineStr">
+        <is>
+          <t>Event reminders, reveal notices, expiry warnings</t>
+        </is>
+      </c>
+      <c r="K32" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>Backlog: Should-have and later phases</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>BL.2</t>
+        </is>
+      </c>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>Backlog: Hall of Fame — Host-curated highlights visible to guests</t>
+        </is>
+      </c>
+      <c r="D33" s="7" t="inlineStr">
+        <is>
+          <t>services/gallery</t>
+        </is>
+      </c>
+      <c r="E33" s="7" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F33" s="7" t="inlineStr"/>
+      <c r="G33" s="7" t="inlineStr"/>
+      <c r="H33" s="7" t="inlineStr"/>
+      <c r="I33" s="7" t="inlineStr">
+        <is>
+          <t>FR-11.1-11.5</t>
+        </is>
+      </c>
+      <c r="J33" s="7" t="inlineStr">
+        <is>
+          <t>Curation, ordering and sharing of the best photos</t>
+        </is>
+      </c>
+      <c r="K33" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="7" t="inlineStr">
+        <is>
+          <t>Backlog: Should-have and later phases</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>BL.3</t>
+        </is>
+      </c>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>Backlog: Personal/Instant Mode (v1.1) — Capture without an event and send results to several recipients</t>
+        </is>
+      </c>
+      <c r="D34" s="7" t="inlineStr">
+        <is>
+          <t>apps/web, services/media</t>
+        </is>
+      </c>
+      <c r="E34" s="7" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F34" s="7" t="inlineStr"/>
+      <c r="G34" s="7" t="inlineStr"/>
+      <c r="H34" s="7" t="inlineStr"/>
+      <c r="I34" s="7" t="inlineStr">
+        <is>
           <t>FR-10.1-10.7</t>
         </is>
       </c>
-      <c r="J32" s="7" t="inlineStr">
+      <c r="J34" s="7" t="inlineStr">
         <is>
           <t>Deferred until Event Mode is stable</t>
         </is>
       </c>
-      <c r="K32" s="7" t="inlineStr">
+      <c r="K34" s="7" t="inlineStr">
         <is>
           <t>2026-09-19</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K32"/>
-  <conditionalFormatting sqref="E2:E32">
+  <autoFilter ref="A1:K34"/>
+  <conditionalFormatting sqref="E2:E34">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$E2="Not Started"</formula>
     </cfRule>
@@ -2670,7 +2792,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="E2:E32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E2:E34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Not Started,In Progress,Pending Verification,Completed"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2684,7 +2806,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2915,37 +3037,37 @@
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>cmd/api</t>
+          <t>apps/web (tests/e2e), scripts</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>T3.7</t>
+          <t>T7.1</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>Wired config, Postgres, Redis, SMTP and the auth service into one process serving HTTP and gRPC, with an end-to-end test.</t>
+          <t>Added Playwright end-to-end tests that drive Chrome through the Vite proxy to the real API, Postgres, Redis and Mailpit (scripts/e2e.sh), and made scripts/check.sh run them; timed the scripted host flow against the 3-minute target.</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>cmd/api's run() now takes (ctx, getenv); the server no longer starts without the required environment.</t>
+          <t>scripts/check.sh now needs Docker (Redis + Mailpit up), Chrome and TEST_DATABASE_URL; SKIP_E2E=1 skips the e2e step with a loud notice. Port 8080 is held by an unrelated Apache service on the dev machine, so e2e uses 8081/9091/5174.</t>
         </is>
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>Services stay packages in one process (deviation from separate deployables, recorded in FSD 2.6). go test -race unavailable locally (needs cgo/gcc); run it in CI.</t>
+          <t>Installed Chrome instead of downloading Playwright browsers; e2e uses a throwaway sela_e2e_&lt;pid&gt; database on the local Postgres and resets only rl:/attempts:/lock: keys on the compose Redis; one unique email per test because of the OTP rate limits; the QR PNG is decoded with jsqr to prove it encodes the short link; scripted time is a lower bound and not the PRD metric. A typescript review found no CRITICAL/HIGH; the MEDIUMs (unguarded database-URL rewrite, unchecked Redis container, one-shot QR load check) were fixed in 7b11984. Also added .gitattributes so shell scripts keep LF.</t>
         </is>
       </c>
       <c r="G6" s="7" t="inlineStr">
         <is>
-          <t>5a3dbe0 2bffd81 578bab2 218243d 573d78f</t>
+          <t>58b435f 56159ff 29d31b5 70c75d0 fcdfe29 44e0983 6037092 d34c798 96d0a2a 7b11984</t>
         </is>
       </c>
       <c r="H6" s="7" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -2957,32 +3079,32 @@
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>cmd/migrate</t>
+          <t>cmd/api</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>T3.1</t>
+          <t>T3.7</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>Added a CLI that applies (up) or reverts (down) migrations against DATABASE_URL.</t>
+          <t>Wired config, Postgres, Redis, SMTP and the auth service into one process serving HTTP and gRPC, with an end-to-end test.</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>None.</t>
+          <t>cmd/api's run() now takes (ctx, getenv); the server no longer starts without the required environment.</t>
         </is>
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>Default command is up; DSN is never printed; run() is injectable for tests.</t>
+          <t>Services stay packages in one process (deviation from separate deployables, recorded in FSD 2.6). go test -race unavailable locally (needs cgo/gcc); run it in CI.</t>
         </is>
       </c>
       <c r="G7" s="7" t="inlineStr">
         <is>
-          <t>f5935c9 a1e047f b2ef0ef</t>
+          <t>5a3dbe0 2bffd81 578bab2 218243d 573d78f</t>
         </is>
       </c>
       <c r="H7" s="7" t="inlineStr">
@@ -2999,17 +3121,17 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>deploy, scripts/check.sh</t>
+          <t>cmd/migrate</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>T1.3</t>
+          <t>T3.1</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>Added Docker Compose services (Postgres, Redis, Mailpit) bound to localhost with required credentials, .env.example and scripts/check.sh.</t>
+          <t>Added a CLI that applies (up) or reverts (down) migrations against DATABASE_URL.</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
@@ -3019,12 +3141,12 @@
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>Compose refuses to start without credentials; check.sh became the single validation entrypoint.</t>
+          <t>Default command is up; DSN is never printed; run() is injectable for tests.</t>
         </is>
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
-          <t>20ade0e cbeb530</t>
+          <t>f5935c9 a1e047f b2ef0ef</t>
         </is>
       </c>
       <c r="H8" s="7" t="inlineStr">
@@ -3041,17 +3163,17 @@
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>docs</t>
+          <t>deploy, cmd/api</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>T3.9</t>
+          <t>T3.8</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>Updated the FSD to v2.5 and created this tracker with its build script and process.</t>
+          <t>Verified the email OTP flow live against docker compose Redis and Mailpit with the real API; all checks passed without service changes.</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
@@ -3061,17 +3183,17 @@
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>PRD and BRD intentionally unchanged: implementation so far does not change product scope, and their documented inconsistencies (MVP category count, free-tier watermark, BR-17 numbering) stay open. docs/ is gitignored, so these updates are not in commits.</t>
+          <t>Verification lives in apps/web/tests/e2e/auth-live.spec.ts so it is repeatable; compose's postgres was not used because a local PostgreSQL 17 owns 5432.</t>
         </is>
       </c>
       <c r="G9" s="7" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>n/a (verification; tests in 44e0983)</t>
         </is>
       </c>
       <c r="H9" s="7" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -3083,17 +3205,17 @@
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>docs</t>
+          <t>deploy, scripts/check.sh</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>T4.4</t>
+          <t>T1.3</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>Updated the FSD to v2.6 and this tracker for Task 4.</t>
+          <t>Added Docker Compose services (Postgres, Redis, Mailpit) bound to localhost with required credentials, .env.example and scripts/check.sh.</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
@@ -3103,17 +3225,17 @@
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>PRD and BRD still unchanged; the fallback defaults are recorded in FSD 4.1 as derived from BRD 7/10 for product review.</t>
+          <t>Compose refuses to start without credentials; check.sh became the single validation entrypoint.</t>
         </is>
       </c>
       <c r="G10" s="7" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>20ade0e cbeb530</t>
         </is>
       </c>
       <c r="H10" s="7" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-19</t>
         </is>
       </c>
     </row>
@@ -3130,12 +3252,12 @@
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>T6.2</t>
+          <t>T3.9</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>Updated the FSD to v2.8 (10.1 implementation note, change row, 11.1 status for FR-01.1, FR-01.2, FR-01.3, FR-09.1), CLAUDE.md and this tracker for Task 6.</t>
+          <t>Updated the FSD to v2.5 and created this tracker with its build script and process.</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
@@ -3145,7 +3267,7 @@
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>FR-01.1 to FR-01.3 are now Completed; FR-09.1 stays Partial (SMS not built, live Redis/SMTP verification pending). Category default numbers remain tbd for product. docs/ is gitignored, so these edits are not versioned.</t>
+          <t>PRD and BRD intentionally unchanged: implementation so far does not change product scope, and their documented inconsistencies (MVP category count, free-tier watermark, BR-17 numbering) stay open. docs/ is gitignored, so these updates are not in commits.</t>
         </is>
       </c>
       <c r="G11" s="7" t="inlineStr">
@@ -3155,7 +3277,7 @@
       </c>
       <c r="H11" s="7" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-19</t>
         </is>
       </c>
     </row>
@@ -3167,37 +3289,37 @@
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>internal/config</t>
+          <t>docs</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>T3.4</t>
+          <t>T4.4</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>Added fail-fast environment loading with aggregated errors and redacted printing.</t>
+          <t>Updated the FSD to v2.6 and this tracker for Task 4.</t>
         </is>
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
-          <t>The API now refuses to start without DATABASE_URL, REDIS_ADDR, SMTP_ADDR, SMTP_FROM and OTP_HMAC_KEY (&gt;= 32 characters).</t>
+          <t>None.</t>
         </is>
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>Secrets never appear in errors or String(); COOKIE_SECURE defaults to true.</t>
+          <t>PRD and BRD still unchanged; the fallback defaults are recorded in FSD 4.1 as derived from BRD 7/10 for product review.</t>
         </is>
       </c>
       <c r="G12" s="7" t="inlineStr">
         <is>
-          <t>730db37 3b1ab82</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="H12" s="7" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -3209,37 +3331,37 @@
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>internal/db</t>
+          <t>docs</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>T2.1</t>
+          <t>T6.2</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>Added the goose migration runner and migrations 0001-0003: hosts, event_categories (six seeded presets) and events.</t>
+          <t>Updated the FSD to v2.8 (10.1 implementation note, change row, 11.1 status for FR-01.1, FR-01.2, FR-01.3, FR-09.1), CLAUDE.md and this tracker for Task 6.</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>New database schema (three migrations). Column names are English forms of FSD 5 (batas_jepretan -&gt; shot_limit, etc.).</t>
+          <t>None.</t>
         </is>
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>Undefined category defaults are stored as 'tbd', never invented. goose pinned to v3.26.0 because v3.28 requires Go 1.26 and silently raised the module's Go version. Cover image and branding columns deferred. Categories are presets, not gates. PII encryption deferred (needs a blind index for the unique lookups).</t>
+          <t>FR-01.1 to FR-01.3 are now Completed; FR-09.1 stays Partial (SMS not built, live Redis/SMTP verification pending). Category default numbers remain tbd for product. docs/ is gitignored, so these edits are not versioned.</t>
         </is>
       </c>
       <c r="G13" s="7" t="inlineStr">
         <is>
-          <t>9fe108b 45b058c b0b5b25</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="H13" s="7" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -3251,32 +3373,32 @@
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>internal/httpx, internal/config, api/proto/v1, services/auth</t>
+          <t>docs</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>T4.3</t>
+          <t>T7.3</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>Extracted the strict JSON body decoder into httpx, added the required SHORT_LINK_BASE_URL setting, extended event.proto, and added a deny-by-default gRPC host interceptor.</t>
+          <t>Updated the FSD to v2.9, CLAUDE.md, the tracking README (timed-check protocol) and this tracker for Task 7.</t>
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
-          <t>SHORT_LINK_BASE_URL is now required at startup (the API refuses to start without it). event.proto changes are additive (new field numbers).</t>
+          <t>None.</t>
         </is>
       </c>
       <c r="F14" s="7" t="inlineStr">
         <is>
-          <t>The auth handlers were refactored onto httpx.DecodeJSON with the existing tests as the safety net. The interceptor reuses the auth package's HostID and error mapping instead of duplicating them.</t>
+          <t>Milestone 1 is complete except T7.2 (human timed sessions), which stays Pending Verification. FR-09.1 stays Partial because SMS OTP is not built. docs/ tracker files are versioned; FSD/PRD/BRD .md and .pdf are still ignored.</t>
         </is>
       </c>
       <c r="G14" s="7" t="inlineStr">
         <is>
-          <t>0a61dd6 3861ee6 1c9b2a8 1110a02 6f8cf8e ff5ae81 b1a51e3 da51888</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="H14" s="7" t="inlineStr">
@@ -3293,32 +3415,32 @@
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>internal/httpx, internal/health, cmd/api</t>
+          <t>internal/config</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>T1.1</t>
+          <t>T3.4</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>Added the shared JSON envelope {success, data, error}, a GET /healthz handler and an HTTP entrypoint with graceful shutdown.</t>
+          <t>Added fail-fast environment loading with aggregated errors and redacted printing.</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>None.</t>
+          <t>The API now refuses to start without DATABASE_URL, REDIS_ADDR, SMTP_ADDR, SMTP_FROM and OTP_HMAC_KEY (&gt;= 32 characters).</t>
         </is>
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>Envelope follows the project API-response rule; health checks no dependencies (liveness only).</t>
+          <t>Secrets never appear in errors or String(); COOKIE_SECURE defaults to true.</t>
         </is>
       </c>
       <c r="G15" s="7" t="inlineStr">
         <is>
-          <t>aae2ee6 bbc37ea 0bd97a3</t>
+          <t>730db37 3b1ab82</t>
         </is>
       </c>
       <c r="H15" s="7" t="inlineStr">
@@ -3335,32 +3457,32 @@
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>services/auth</t>
+          <t>internal/db</t>
         </is>
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>T3.5</t>
+          <t>T2.1</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>Implemented the OTP sign-in core: hashed single-use 5-minute codes, rate limits, lockout, hashed 12-hour sessions, Postgres find-or-create host and an SMTP mailer.</t>
+          <t>Added the goose migration runner and migrations 0001-0003: hosts, event_categories (six seeded presets) and events.</t>
         </is>
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
-          <t>Adds runtime dependencies on Redis and an SMTP relay.</t>
+          <t>New database schema (three migrations). Column names are English forms of FSD 5 (batas_jepretan -&gt; shot_limit, etc.).</t>
         </is>
       </c>
       <c r="F16" s="7" t="inlineStr">
         <is>
-          <t>Code consumed before host creation so concurrent verifies cannot mis-report IsNewHost; attempts counted only while a code is outstanding to prevent lockout of addresses that never requested a code; Redis keys use keyed hashes (no raw email or IP); opaque server-side sessions instead of JWT; refresh token and logout deferred (partial FR-SEC.4).</t>
+          <t>Undefined category defaults are stored as 'tbd', never invented. goose pinned to v3.26.0 because v3.28 requires Go 1.26 and silently raised the module's Go version. Cover image and branding columns deferred. Categories are presets, not gates. PII encryption deferred (needs a blind index for the unique lookups).</t>
         </is>
       </c>
       <c r="G16" s="7" t="inlineStr">
         <is>
-          <t>1043ded 3c45e13</t>
+          <t>9fe108b 45b058c b0b5b25</t>
         </is>
       </c>
       <c r="H16" s="7" t="inlineStr">
@@ -3377,37 +3499,37 @@
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>services/auth</t>
+          <t>internal/httpx, internal/config, api/proto/v1, services/auth</t>
         </is>
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>T3.6</t>
+          <t>T4.3</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>Added REST and gRPC adapters over one Flow interface, plus RequireHost middleware.</t>
+          <t>Extracted the strict JSON body decoder into httpx, added the required SHORT_LINK_BASE_URL setting, extended event.proto, and added a deny-by-default gRPC host interceptor.</t>
         </is>
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
-          <t>None.</t>
+          <t>SHORT_LINK_BASE_URL is now required at startup (the API refuses to start without it). event.proto changes are additive (new field numbers).</t>
         </is>
       </c>
       <c r="F17" s="7" t="inlineStr">
         <is>
-          <t>HTTP handlers live in services/auth (not internal/httpx), reusing the httpx envelope. Session token only in the HttpOnly cookie (HTTP) or the response (gRPC). X-Forwarded-For deliberately ignored. Fixed generic messages for internal errors.</t>
+          <t>The auth handlers were refactored onto httpx.DecodeJSON with the existing tests as the safety net. The interceptor reuses the auth package's HostID and error mapping instead of duplicating them.</t>
         </is>
       </c>
       <c r="G17" s="7" t="inlineStr">
         <is>
-          <t>ffed71f ce4729e</t>
+          <t>0a61dd6 3861ee6 1c9b2a8 1110a02 6f8cf8e ff5ae81 b1a51e3 da51888</t>
         </is>
       </c>
       <c r="H17" s="7" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -3419,37 +3541,37 @@
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>services/event</t>
+          <t>internal/httpx, internal/health, cmd/api</t>
         </is>
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>T4.1</t>
+          <t>T1.1</t>
         </is>
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>Added the event domain: category presets with raw and effective defaults, event creation with unique short codes and private access tokens, PNG/SVG QR codes of the short link, and host-scoped retrieval.</t>
+          <t>Added the shared JSON envelope {success, data, error}, a GET /healthz handler and an HTTP entrypoint with graceful shutdown.</t>
         </is>
       </c>
       <c r="E18" s="7" t="inlineStr">
         <is>
-          <t>None to existing endpoints; new tables are read and written (events, event_categories) with no schema change.</t>
+          <t>None.</t>
         </is>
       </c>
       <c r="F18" s="7" t="inlineStr">
         <is>
-          <t>FSD does not define what a tbd default falls back to, so the fallback is unlimited shots and instant reveal, derived from BRD 7/10 and FSD 4.5. Host override beats a defined category default beats the fallback. Wedding reveal_at = start of the event day (Asia/Jakarta) + 24h, an interpretation of 'delayed 1 day' that needs product confirmation. shot_limit 0 means explicitly unlimited. reveal_delay_hours capped at 8760 (safety limit, not in the docs). Not-owner and not-found are both ErrNotFound so existence is not leaked. Timezone data is embedded (time/tzdata). Short-link resolver deliberately deferred.</t>
+          <t>Envelope follows the project API-response rule; health checks no dependencies (liveness only).</t>
         </is>
       </c>
       <c r="G18" s="7" t="inlineStr">
         <is>
-          <t>acbece7 b726530</t>
+          <t>aae2ee6 bbc37ea 0bd97a3</t>
         </is>
       </c>
       <c r="H18" s="7" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-19</t>
         </is>
       </c>
     </row>
@@ -3461,37 +3583,37 @@
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>services/event</t>
+          <t>services/auth</t>
         </is>
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>T5.1</t>
+          <t>T3.5</t>
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>Added the public short-link resolver GET /e/{short_code} returning guest-safe event metadata; short links and QR codes now encode {SHORT_LINK_BASE_URL}/e/{code}.</t>
+          <t>Implemented the OTP sign-in core: hashed single-use 5-minute codes, rate limits, lockout, hashed 12-hour sessions, Postgres find-or-create host and an SMTP mailer.</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr">
         <is>
-          <t>Short links/QR codes created before this change lack /e/ (dev/test data only).</t>
+          <t>Adds runtime dependencies on Redis and an SMTP relay.</t>
         </is>
       </c>
       <c r="F19" s="7" t="inlineStr">
         <is>
-          <t>Invalid, unknown, non-active and expired codes all return one identical 404; 200 JSON rather than a redirect (no guest PWA yet); no rate limiting yet (follow-up); no proto change.</t>
+          <t>Code consumed before host creation so concurrent verifies cannot mis-report IsNewHost; attempts counted only while a code is outstanding to prevent lockout of addresses that never requested a code; Redis keys use keyed hashes (no raw email or IP); opaque server-side sessions instead of JWT; refresh token and logout deferred (partial FR-SEC.4).</t>
         </is>
       </c>
       <c r="G19" s="7" t="inlineStr">
         <is>
-          <t>1c6b579 4a9208e 1c6fa33 97bdbe1 e8c01ae 0e537e9 bebb849</t>
+          <t>1043ded 3c45e13</t>
         </is>
       </c>
       <c r="H19" s="7" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-19</t>
         </is>
       </c>
     </row>
@@ -3503,42 +3625,168 @@
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
+          <t>services/auth</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>T3.6</t>
+        </is>
+      </c>
+      <c r="D20" s="7" t="inlineStr">
+        <is>
+          <t>Added REST and gRPC adapters over one Flow interface, plus RequireHost middleware.</t>
+        </is>
+      </c>
+      <c r="E20" s="7" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+      <c r="F20" s="7" t="inlineStr">
+        <is>
+          <t>HTTP handlers live in services/auth (not internal/httpx), reusing the httpx envelope. Session token only in the HttpOnly cookie (HTTP) or the response (gRPC). X-Forwarded-For deliberately ignored. Fixed generic messages for internal errors.</t>
+        </is>
+      </c>
+      <c r="G20" s="7" t="inlineStr">
+        <is>
+          <t>ffed71f ce4729e</t>
+        </is>
+      </c>
+      <c r="H20" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>Milestone 1: Host creates an event</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>services/event</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>T4.1</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="inlineStr">
+        <is>
+          <t>Added the event domain: category presets with raw and effective defaults, event creation with unique short codes and private access tokens, PNG/SVG QR codes of the short link, and host-scoped retrieval.</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="inlineStr">
+        <is>
+          <t>None to existing endpoints; new tables are read and written (events, event_categories) with no schema change.</t>
+        </is>
+      </c>
+      <c r="F21" s="7" t="inlineStr">
+        <is>
+          <t>FSD does not define what a tbd default falls back to, so the fallback is unlimited shots and instant reveal, derived from BRD 7/10 and FSD 4.5. Host override beats a defined category default beats the fallback. Wedding reveal_at = start of the event day (Asia/Jakarta) + 24h, an interpretation of 'delayed 1 day' that needs product confirmation. shot_limit 0 means explicitly unlimited. reveal_delay_hours capped at 8760 (safety limit, not in the docs). Not-owner and not-found are both ErrNotFound so existence is not leaked. Timezone data is embedded (time/tzdata). Short-link resolver deliberately deferred.</t>
+        </is>
+      </c>
+      <c r="G21" s="7" t="inlineStr">
+        <is>
+          <t>acbece7 b726530</t>
+        </is>
+      </c>
+      <c r="H21" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>Milestone 1: Host creates an event</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>services/event</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>T5.1</t>
+        </is>
+      </c>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>Added the public short-link resolver GET /e/{short_code} returning guest-safe event metadata; short links and QR codes now encode {SHORT_LINK_BASE_URL}/e/{code}.</t>
+        </is>
+      </c>
+      <c r="E22" s="7" t="inlineStr">
+        <is>
+          <t>Short links/QR codes created before this change lack /e/ (dev/test data only).</t>
+        </is>
+      </c>
+      <c r="F22" s="7" t="inlineStr">
+        <is>
+          <t>Invalid, unknown, non-active and expired codes all return one identical 404; 200 JSON rather than a redirect (no guest PWA yet); no rate limiting yet (follow-up); no proto change.</t>
+        </is>
+      </c>
+      <c r="G22" s="7" t="inlineStr">
+        <is>
+          <t>1c6b579 4a9208e 1c6fa33 97bdbe1 e8c01ae 0e537e9 bebb849</t>
+        </is>
+      </c>
+      <c r="H22" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>Milestone 1: Host creates an event</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
           <t>services/event, cmd/api</t>
         </is>
       </c>
-      <c r="C20" s="7" t="inlineStr">
+      <c r="C23" s="7" t="inlineStr">
         <is>
           <t>T4.2</t>
         </is>
       </c>
-      <c r="D20" s="7" t="inlineStr">
+      <c r="D23" s="7" t="inlineStr">
         <is>
           <t>Exposed the event use cases over REST and gRPC and wired them into the API process.</t>
         </is>
       </c>
-      <c r="E20" s="7" t="inlineStr">
+      <c r="E23" s="7" t="inlineStr">
         <is>
           <t>cmd/api's newMux and newGRPCServer now take the event dependencies; the gRPC server always installs the host interceptor, so every method outside the public allowlist requires a Bearer session.</t>
         </is>
       </c>
-      <c r="F20" s="7" t="inlineStr">
+      <c r="F23" s="7" t="inlineStr">
         <is>
           <t>Category listing is public (presets, not host data); everything else needs a session. The RPC keeps the name ListEventCategories (existing contract) instead of ListCategories. Responses are built from types that have no host_id or access_token field, and request bodies containing host_id are rejected. HTTP handlers live in services/event and reuse the httpx envelope. golangci-lint timeout raised to 5 minutes in check.sh.</t>
         </is>
       </c>
-      <c r="G20" s="7" t="inlineStr">
+      <c r="G23" s="7" t="inlineStr">
         <is>
           <t>6c65e04 094e6bb aeb1251 cb7f51b 51a1ef0</t>
         </is>
       </c>
-      <c r="H20" s="7" t="inlineStr">
+      <c r="H23" s="7" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H20"/>
+  <autoFilter ref="A1:H23"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4623,12 +4871,12 @@
       </c>
       <c r="F35" s="7" t="inlineStr">
         <is>
-          <t>T3.3, T3.5, T3.6, T3.7, T3.8, T6.1</t>
+          <t>T3.3, T3.5, T3.6, T3.7, T3.8, T6.1, T7.1</t>
         </is>
       </c>
       <c r="G35" s="7" t="inlineStr">
         <is>
-          <t>email OTP over REST and gRPC; host sign-in page /auth/login (two steps, localised errors, rate-limit and lockout wait); SMS not implemented; live-infra verification pending</t>
+          <t>email OTP over REST and gRPC; host sign-in page /auth/login (two steps, localised errors, rate-limit and lockout wait); verified live against real Redis and Mailpit (T3.8, T7.1); SMS not implemented</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: record Task 8.1 (guest session and media schema) in the tracker
T8.1 is Pending Verification: RED 6d1e157, GREEN 720b11f. The schema tests
were mirrored against PostgreSQL 16 and type-checked, but scripts/check.sh
has not run on this change yet. FR-02.2 marked Partial. The FSD moves to
v2.10 with Section 5 notes for migration 0004 (the FSD is kept outside git).

FR-02.2

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012q8YVM7WcTSqottbYMNx19
</commit_message>
<xml_diff>
--- a/docs/tracking/SELA_Progress_Tracker.xlsx
+++ b/docs/tracking/SELA_Progress_Tracker.xlsx
@@ -14,8 +14,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Tracker'!$A$1:$K$34</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Change Log'!$A$1:$H$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Tracker'!$A$1:$K$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Change Log'!$A$1:$H$25</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Traceability'!$A$1:$G$59</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -516,7 +516,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Data as of 2026-09-19. Generated from docs/tracking/tracker.json and docs/FSD_Sela.md; do not edit this workbook by hand.</t>
+          <t>Data as of 2026-09-23. Generated from docs/tracking/tracker.json and docs/FSD_Sela.md; do not edit this workbook by hand.</t>
         </is>
       </c>
     </row>
@@ -982,7 +982,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K34"/>
+  <dimension ref="A1:K35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2419,67 +2419,79 @@
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
         <is>
-          <t>Milestone 3: Role-correct gallery</t>
+          <t>Milestone 2: Guest captures and uploads</t>
         </is>
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>M3.1</t>
+          <t>T8.1</t>
         </is>
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>Milestone 3 (not yet planned) — Role-correct gallery, reveal timer, real-time channels</t>
+          <t>Task 8: Guest session and media schema — Migration 0004 (guest_sessions, media, events.involves_minors) and the services/media domain types</t>
         </is>
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>services/gallery, services/realtime</t>
+          <t>internal/db, services/media</t>
         </is>
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F27" s="7" t="inlineStr"/>
-      <c r="G27" s="7" t="inlineStr"/>
-      <c r="H27" s="7" t="inlineStr"/>
+          <t>Pending Verification</t>
+        </is>
+      </c>
+      <c r="F27" s="7" t="inlineStr">
+        <is>
+          <t>6d1e157</t>
+        </is>
+      </c>
+      <c r="G27" s="7" t="inlineStr">
+        <is>
+          <t>720b11f</t>
+        </is>
+      </c>
+      <c r="H27" s="7" t="inlineStr">
+        <is>
+          <t>100% (services/media)</t>
+        </is>
+      </c>
       <c r="I27" s="7" t="inlineStr">
         <is>
-          <t>FR-05.1-05.6</t>
+          <t>FR-02.2, FR-04.1, FR-05.5, FR-05.6</t>
         </is>
       </c>
       <c r="J27" s="7" t="inlineStr">
         <is>
-          <t>Host sees all media, guest only their own, WebSocket channels split by role</t>
+          <t>Schema with the same-event session key, Hall of Fame rules and gallery indexes. Open: the Go schema tests were mirrored against Postgres 16 (49/49) and type-checked, but scripts/check.sh has not run on this change yet</t>
         </is>
       </c>
       <c r="K27" s="7" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>Milestone 4: Moderate and export</t>
+          <t>Milestone 3: Role-correct gallery</t>
         </is>
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>M4.1</t>
+          <t>M3.1</t>
         </is>
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>Milestone 4 (not yet planned) — Moderation and full-gallery ZIP export</t>
+          <t>Milestone 3 (not yet planned) — Role-correct gallery, reveal timer, real-time channels</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>services/gallery, services/media</t>
+          <t>services/gallery, services/realtime</t>
         </is>
       </c>
       <c r="E28" s="7" t="inlineStr">
@@ -2492,12 +2504,12 @@
       <c r="H28" s="7" t="inlineStr"/>
       <c r="I28" s="7" t="inlineStr">
         <is>
-          <t>FR-06.1-06.4, FR-07.1-07.3</t>
+          <t>FR-05.1-05.6</t>
         </is>
       </c>
       <c r="J28" s="7" t="inlineStr">
         <is>
-          <t>Hide/delete, asynchronous ZIP export, share links</t>
+          <t>Host sees all media, guest only their own, WebSocket channels split by role</t>
         </is>
       </c>
       <c r="K28" s="7" t="inlineStr">
@@ -2509,22 +2521,22 @@
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
         <is>
-          <t>Milestone 5: Plans and payment</t>
+          <t>Milestone 4: Moderate and export</t>
         </is>
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>M5.1</t>
+          <t>M4.1</t>
         </is>
       </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>Milestone 5 (not yet planned) — Plans, package recommendation and payment (QRIS, e-wallet, card)</t>
+          <t>Milestone 4 (not yet planned) — Moderation and full-gallery ZIP export</t>
         </is>
       </c>
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>services/payment, services/event</t>
+          <t>services/gallery, services/media</t>
         </is>
       </c>
       <c r="E29" s="7" t="inlineStr">
@@ -2537,12 +2549,12 @@
       <c r="H29" s="7" t="inlineStr"/>
       <c r="I29" s="7" t="inlineStr">
         <is>
-          <t>FR-01.5, FR-01.6, FR-09.2, FR-09.3</t>
+          <t>FR-06.1-06.4, FR-07.1-07.3</t>
         </is>
       </c>
       <c r="J29" s="7" t="inlineStr">
         <is>
-          <t>Free and paid tiers by event scale; micro-payments; transaction history</t>
+          <t>Hide/delete, asynchronous ZIP export, share links</t>
         </is>
       </c>
       <c r="K29" s="7" t="inlineStr">
@@ -2554,22 +2566,22 @@
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
         <is>
-          <t>Milestone 6: Privacy and compliance readiness</t>
+          <t>Milestone 5: Plans and payment</t>
         </is>
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>M6.1</t>
+          <t>M5.1</t>
         </is>
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>Milestone 6 (not yet planned) — Privacy and compliance readiness</t>
+          <t>Milestone 5 (not yet planned) — Plans, package recommendation and payment (QRIS, e-wallet, card)</t>
         </is>
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>cross-cutting</t>
+          <t>services/payment, services/event</t>
         </is>
       </c>
       <c r="E30" s="7" t="inlineStr">
@@ -2582,12 +2594,12 @@
       <c r="H30" s="7" t="inlineStr"/>
       <c r="I30" s="7" t="inlineStr">
         <is>
-          <t>FR-SEC.1, FR-SEC.5-SEC.8, FR-SEC.10</t>
+          <t>FR-01.5, FR-01.6, FR-09.2, FR-09.3</t>
         </is>
       </c>
       <c r="J30" s="7" t="inlineStr">
         <is>
-          <t>PII column encryption with a blind index, audit log, retention and deletion, child-event defaults, noindex headers</t>
+          <t>Free and paid tiers by event scale; micro-payments; transaction history</t>
         </is>
       </c>
       <c r="K30" s="7" t="inlineStr">
@@ -2599,22 +2611,22 @@
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
         <is>
-          <t>Milestone 7: Closed beta</t>
+          <t>Milestone 6: Privacy and compliance readiness</t>
         </is>
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>M7.1</t>
+          <t>M6.1</t>
         </is>
       </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
-          <t>Milestone 7 (not yet planned) — Closed beta across wedding, graduation and birthday events</t>
+          <t>Milestone 6 (not yet planned) — Privacy and compliance readiness</t>
         </is>
       </c>
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>operations</t>
+          <t>cross-cutting</t>
         </is>
       </c>
       <c r="E31" s="7" t="inlineStr">
@@ -2625,10 +2637,14 @@
       <c r="F31" s="7" t="inlineStr"/>
       <c r="G31" s="7" t="inlineStr"/>
       <c r="H31" s="7" t="inlineStr"/>
-      <c r="I31" s="7" t="inlineStr"/>
+      <c r="I31" s="7" t="inlineStr">
+        <is>
+          <t>FR-SEC.1, FR-SEC.5-SEC.8, FR-SEC.10</t>
+        </is>
+      </c>
       <c r="J31" s="7" t="inlineStr">
         <is>
-          <t>Validate the hypothesis and fill the TBD success metrics in the PRD</t>
+          <t>PII column encryption with a blind index, audit log, retention and deletion, child-event defaults, noindex headers</t>
         </is>
       </c>
       <c r="K31" s="7" t="inlineStr">
@@ -2640,22 +2656,22 @@
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
         <is>
-          <t>Backlog: Should-have and later phases</t>
+          <t>Milestone 7: Closed beta</t>
         </is>
       </c>
       <c r="B32" s="7" t="inlineStr">
         <is>
-          <t>BL.1</t>
+          <t>M7.1</t>
         </is>
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>Backlog: Notifications — Scheduled and transactional email/WhatsApp notifications</t>
+          <t>Milestone 7 (not yet planned) — Closed beta across wedding, graduation and birthday events</t>
         </is>
       </c>
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>services/notification</t>
+          <t>operations</t>
         </is>
       </c>
       <c r="E32" s="7" t="inlineStr">
@@ -2666,14 +2682,10 @@
       <c r="F32" s="7" t="inlineStr"/>
       <c r="G32" s="7" t="inlineStr"/>
       <c r="H32" s="7" t="inlineStr"/>
-      <c r="I32" s="7" t="inlineStr">
-        <is>
-          <t>FR-08.1-08.2</t>
-        </is>
-      </c>
+      <c r="I32" s="7" t="inlineStr"/>
       <c r="J32" s="7" t="inlineStr">
         <is>
-          <t>Event reminders, reveal notices, expiry warnings</t>
+          <t>Validate the hypothesis and fill the TBD success metrics in the PRD</t>
         </is>
       </c>
       <c r="K32" s="7" t="inlineStr">
@@ -2690,17 +2702,17 @@
       </c>
       <c r="B33" s="7" t="inlineStr">
         <is>
-          <t>BL.2</t>
+          <t>BL.1</t>
         </is>
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>Backlog: Hall of Fame — Host-curated highlights visible to guests</t>
+          <t>Backlog: Notifications — Scheduled and transactional email/WhatsApp notifications</t>
         </is>
       </c>
       <c r="D33" s="7" t="inlineStr">
         <is>
-          <t>services/gallery</t>
+          <t>services/notification</t>
         </is>
       </c>
       <c r="E33" s="7" t="inlineStr">
@@ -2713,12 +2725,12 @@
       <c r="H33" s="7" t="inlineStr"/>
       <c r="I33" s="7" t="inlineStr">
         <is>
-          <t>FR-11.1-11.5</t>
+          <t>FR-08.1-08.2</t>
         </is>
       </c>
       <c r="J33" s="7" t="inlineStr">
         <is>
-          <t>Curation, ordering and sharing of the best photos</t>
+          <t>Event reminders, reveal notices, expiry warnings</t>
         </is>
       </c>
       <c r="K33" s="7" t="inlineStr">
@@ -2735,17 +2747,17 @@
       </c>
       <c r="B34" s="7" t="inlineStr">
         <is>
-          <t>BL.3</t>
+          <t>BL.2</t>
         </is>
       </c>
       <c r="C34" s="7" t="inlineStr">
         <is>
-          <t>Backlog: Personal/Instant Mode (v1.1) — Capture without an event and send results to several recipients</t>
+          <t>Backlog: Hall of Fame — Host-curated highlights visible to guests</t>
         </is>
       </c>
       <c r="D34" s="7" t="inlineStr">
         <is>
-          <t>apps/web, services/media</t>
+          <t>services/gallery</t>
         </is>
       </c>
       <c r="E34" s="7" t="inlineStr">
@@ -2758,23 +2770,68 @@
       <c r="H34" s="7" t="inlineStr"/>
       <c r="I34" s="7" t="inlineStr">
         <is>
+          <t>FR-11.1-11.5</t>
+        </is>
+      </c>
+      <c r="J34" s="7" t="inlineStr">
+        <is>
+          <t>Curation, ordering and sharing of the best photos</t>
+        </is>
+      </c>
+      <c r="K34" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="7" t="inlineStr">
+        <is>
+          <t>Backlog: Should-have and later phases</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>BL.3</t>
+        </is>
+      </c>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>Backlog: Personal/Instant Mode (v1.1) — Capture without an event and send results to several recipients</t>
+        </is>
+      </c>
+      <c r="D35" s="7" t="inlineStr">
+        <is>
+          <t>apps/web, services/media</t>
+        </is>
+      </c>
+      <c r="E35" s="7" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F35" s="7" t="inlineStr"/>
+      <c r="G35" s="7" t="inlineStr"/>
+      <c r="H35" s="7" t="inlineStr"/>
+      <c r="I35" s="7" t="inlineStr">
+        <is>
           <t>FR-10.1-10.7</t>
         </is>
       </c>
-      <c r="J34" s="7" t="inlineStr">
+      <c r="J35" s="7" t="inlineStr">
         <is>
           <t>Deferred until Event Mode is stable</t>
         </is>
       </c>
-      <c r="K34" s="7" t="inlineStr">
+      <c r="K35" s="7" t="inlineStr">
         <is>
           <t>2026-09-19</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K34"/>
-  <conditionalFormatting sqref="E2:E34">
+  <autoFilter ref="A1:K35"/>
+  <conditionalFormatting sqref="E2:E35">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$E2="Not Started"</formula>
     </cfRule>
@@ -2792,7 +2849,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="E2:E34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E2:E35" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Not Started,In Progress,Pending Verification,Completed"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2806,7 +2863,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H23"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3785,8 +3842,92 @@
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>Milestone 2: Guest captures and uploads</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>T8.1</t>
+        </is>
+      </c>
+      <c r="D24" s="7" t="inlineStr">
+        <is>
+          <t>Updated the FSD to v2.10 (Section 5 implementation notes for migration 0004) and this tracker.</t>
+        </is>
+      </c>
+      <c r="E24" s="7" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+      <c r="F24" s="7" t="inlineStr">
+        <is>
+          <t>Guest visibility stays as FSD 3.2 and 4.5 define it (own media, plus the Hall of Fame after reveal); the gallery queries come in a later task.</t>
+        </is>
+      </c>
+      <c r="G24" s="7" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H24" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>Milestone 2: Guest captures and uploads</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>internal/db, services/media</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>T8.1</t>
+        </is>
+      </c>
+      <c r="D25" s="7" t="inlineStr">
+        <is>
+          <t>Added migration 0004: guest_sessions, media and events.involves_minors, with schema tests and the media domain types.</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>New migration 0004 (additive). events gains involves_minors boolean NOT NULL DEFAULT false.</t>
+        </is>
+      </c>
+      <c r="F25" s="7" t="inlineStr">
+        <is>
+          <t>No sisa_jepretan column (Redis holds the live counter; the durable count comes from media rows). No browser fingerprint (FSD 8.11 data minimisation). processing_state is separate from the moderation status. The composite key media.(event_id, session_id) -&gt; guest_sessions keeps a session inside its own event. RESTRICT deletes, so the retention job removes stored objects first. WebP accepted beside the FR-04.1 formats because the camera pipeline outputs it (FSD 7).</t>
+        </is>
+      </c>
+      <c r="G25" s="7" t="inlineStr">
+        <is>
+          <t>6d1e157 720b11f</t>
+        </is>
+      </c>
+      <c r="H25" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H23"/>
+  <autoFilter ref="A1:H25"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4112,11 +4253,19 @@
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F9" s="7" t="inlineStr"/>
-      <c r="G9" s="7" t="inlineStr"/>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>T8.1</t>
+        </is>
+      </c>
+      <c r="G9" s="7" t="inlineStr">
+        <is>
+          <t>guest_sessions table (one row per device session, optional nickname, no fingerprint); session creation and the guest cookie are not built yet</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">

</xml_diff>

<commit_message>
docs: update the SELA progress tracker
Co-Authored-By: Claude Code <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/tracking/SELA_Progress_Tracker.xlsx
+++ b/docs/tracking/SELA_Progress_Tracker.xlsx
@@ -14,8 +14,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Tracker'!$A$1:$K$34</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Change Log'!$A$1:$H$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Tracker'!$A$1:$K$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Change Log'!$A$1:$H$26</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Traceability'!$A$1:$G$59</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -516,7 +516,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Data as of 2026-09-19. Generated from docs/tracking/tracker.json and docs/FSD_Sela.md; do not edit this workbook by hand.</t>
+          <t>Data as of 2026-09-23. Generated from docs/tracking/tracker.json and docs/FSD_Sela.md; do not edit this workbook by hand.</t>
         </is>
       </c>
     </row>
@@ -593,7 +593,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -862,7 +862,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Backlog: Should-have and later phases</t>
+          <t>Milestone 8: RBAC foundation (cross-cutting platform work)</t>
         </is>
       </c>
       <c r="B9">
@@ -893,27 +893,27 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>All tasks</t>
+          <t>Backlog: Should-have and later phases</t>
         </is>
       </c>
       <c r="B10">
-        <f>SUM(B2:B9)</f>
+        <f>COUNTIFS(Tracker!$A:$A,$A10,Tracker!$E:$E,B$1)</f>
         <v/>
       </c>
       <c r="C10">
-        <f>SUM(C2:C9)</f>
+        <f>COUNTIFS(Tracker!$A:$A,$A10,Tracker!$E:$E,C$1)</f>
         <v/>
       </c>
       <c r="D10">
-        <f>SUM(D2:D9)</f>
+        <f>COUNTIFS(Tracker!$A:$A,$A10,Tracker!$E:$E,D$1)</f>
         <v/>
       </c>
       <c r="E10">
-        <f>SUM(E2:E9)</f>
+        <f>COUNTIFS(Tracker!$A:$A,$A10,Tracker!$E:$E,E$1)</f>
         <v/>
       </c>
       <c r="F10">
-        <f>SUM(F2:F9)</f>
+        <f>SUM(B10:E10)</f>
         <v/>
       </c>
       <c r="G10" s="5">
@@ -921,53 +921,84 @@
         <v/>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>All tasks</t>
+        </is>
+      </c>
+      <c r="B11">
+        <f>SUM(B2:B10)</f>
+        <v/>
+      </c>
+      <c r="C11">
+        <f>SUM(C2:C10)</f>
+        <v/>
+      </c>
+      <c r="D11">
+        <f>SUM(D2:D10)</f>
+        <v/>
+      </c>
+      <c r="E11">
+        <f>SUM(E2:E10)</f>
+        <v/>
+      </c>
+      <c r="F11">
+        <f>SUM(F2:F10)</f>
+        <v/>
+      </c>
+      <c r="G11" s="5">
+        <f>IF(F11=0,0,E11/F11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>Requirements (FR IDs)</t>
         </is>
       </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
         <is>
           <t>Partial</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
+      <c r="D13" s="4" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="E12" s="4" t="inlineStr">
+      <c r="E13" s="4" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>All FR IDs</t>
         </is>
       </c>
-      <c r="B13">
-        <f>COUNTIF(Traceability!$E:$E,B12)</f>
-        <v/>
-      </c>
-      <c r="C13">
-        <f>COUNTIF(Traceability!$E:$E,C12)</f>
-        <v/>
-      </c>
-      <c r="D13">
-        <f>COUNTIF(Traceability!$E:$E,D12)</f>
-        <v/>
-      </c>
-      <c r="E13">
-        <f>SUM(B13:D13)</f>
+      <c r="B14">
+        <f>COUNTIF(Traceability!$E:$E,B13)</f>
+        <v/>
+      </c>
+      <c r="C14">
+        <f>COUNTIF(Traceability!$E:$E,C13)</f>
+        <v/>
+      </c>
+      <c r="D14">
+        <f>COUNTIF(Traceability!$E:$E,D13)</f>
+        <v/>
+      </c>
+      <c r="E14">
+        <f>SUM(B14:D14)</f>
         <v/>
       </c>
     </row>
@@ -982,7 +1013,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K34"/>
+  <dimension ref="A1:K37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2640,141 +2671,300 @@
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
         <is>
-          <t>Backlog: Should-have and later phases</t>
+          <t>Milestone 8: RBAC foundation (cross-cutting platform work)</t>
         </is>
       </c>
       <c r="B32" s="7" t="inlineStr">
         <is>
-          <t>BL.1</t>
+          <t>T9.1</t>
         </is>
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>Backlog: Notifications — Scheduled and transactional email/WhatsApp notifications</t>
+          <t>Task 9: RBAC foundation — RBAC schema (roles, menus, dropdowns, actions/permissions) and the services/rbac backend package; events:create gated on the already-shipped create-event route</t>
         </is>
       </c>
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>services/notification</t>
+          <t>internal/db (0004, 0005), services/rbac, services/event, cmd/api</t>
         </is>
       </c>
       <c r="E32" s="7" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F32" s="7" t="inlineStr"/>
-      <c r="G32" s="7" t="inlineStr"/>
-      <c r="H32" s="7" t="inlineStr"/>
-      <c r="I32" s="7" t="inlineStr">
-        <is>
-          <t>FR-08.1-08.2</t>
-        </is>
-      </c>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F32" s="7" t="inlineStr">
+        <is>
+          <t>85ac425 e76992d 08d0812 68ae150</t>
+        </is>
+      </c>
+      <c r="G32" s="7" t="inlineStr">
+        <is>
+          <t>cf5f3a8 b85cbb8 1bc1ec4 bb79173</t>
+        </is>
+      </c>
+      <c r="H32" s="7" t="inlineStr">
+        <is>
+          <t>services/rbac 81.9%; services/event 91.3%; cmd/api 83.3%</t>
+        </is>
+      </c>
+      <c r="I32" s="7" t="inlineStr"/>
       <c r="J32" s="7" t="inlineStr">
         <is>
-          <t>Event reminders, reveal notices, expiry warnings</t>
+          <t>migrations 0004_rbac_foundation.sql, 0005_hosts_role_and_preferences.sql; services/rbac (types/postgres/service/http) with GET /api/v1/auth/me and PATCH /api/v1/me/preferences; RequirePermission wired onto POST /api/v1/events (events:create); seed limited to 2 menus (events_new, settings) and 2 enforced permissions (events:create, profile:update), every existing host granted both so no current behavior changes</t>
         </is>
       </c>
       <c r="K32" s="7" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
         <is>
-          <t>Backlog: Should-have and later phases</t>
+          <t>Milestone 8: RBAC foundation (cross-cutting platform work)</t>
         </is>
       </c>
       <c r="B33" s="7" t="inlineStr">
         <is>
-          <t>BL.2</t>
+          <t>T9.2</t>
         </is>
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>Backlog: Hall of Fame — Host-curated highlights visible to guests</t>
+          <t>Task 9: RBAC foundation — Frontend: rbac API client, best-effort profile fetch in the root layout, dynamic Nav, dark theme palette, and the new /settings page with real EN/ID switching</t>
         </is>
       </c>
       <c r="D33" s="7" t="inlineStr">
         <is>
-          <t>services/gallery</t>
+          <t>apps/web</t>
         </is>
       </c>
       <c r="E33" s="7" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F33" s="7" t="inlineStr"/>
-      <c r="G33" s="7" t="inlineStr"/>
-      <c r="H33" s="7" t="inlineStr"/>
-      <c r="I33" s="7" t="inlineStr">
-        <is>
-          <t>FR-11.1-11.5</t>
-        </is>
-      </c>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F33" s="7" t="inlineStr">
+        <is>
+          <t>14bc5fe 6dea65a 4be3c95</t>
+        </is>
+      </c>
+      <c r="G33" s="7" t="inlineStr">
+        <is>
+          <t>21fbdb5 e1cb469 23963e0 d98a473 694ba26 99c2c86</t>
+        </is>
+      </c>
+      <c r="H33" s="7" t="inlineStr">
+        <is>
+          <t>184 tests pass; 97.16% statements / 89.65% branches / 97.6% functions / 99.75% lines; svelte-check 0 errors/0 warnings</t>
+        </is>
+      </c>
+      <c r="I33" s="7" t="inlineStr"/>
       <c r="J33" s="7" t="inlineStr">
         <is>
-          <t>Curation, ordering and sharing of the best photos</t>
+          <t>src/lib/api/rbac.ts; src/lib/components/Nav.svelte; :root[data-theme='dark'] palette in tokens.css; +layout.ts best-effort getProfile() (swallows a 401 so /auth/login never breaks); +layout.svelte renders Nav and sets document.documentElement.dataset.theme; src/routes/settings/+page.svelte (role, theme toggle, language toggle, own local EN/ID string table); the three pre-existing host pages keep their hardcoded Indonesian text unchanged</t>
         </is>
       </c>
       <c r="K33" s="7" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
         <is>
+          <t>Milestone 8: RBAC foundation (cross-cutting platform work)</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>T9.3</t>
+        </is>
+      </c>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>Task 9: RBAC foundation — Real-stack verification and docs/tracking sync for Task 8</t>
+        </is>
+      </c>
+      <c r="D34" s="7" t="inlineStr">
+        <is>
+          <t>docs, docs/tracking, CLAUDE.md</t>
+        </is>
+      </c>
+      <c r="E34" s="7" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F34" s="7" t="inlineStr">
+        <is>
+          <t>n/a (documentation)</t>
+        </is>
+      </c>
+      <c r="G34" s="7" t="inlineStr">
+        <is>
+          <t>n/a (docs/ is gitignored, not committed)</t>
+        </is>
+      </c>
+      <c r="H34" s="7" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I34" s="7" t="inlineStr"/>
+      <c r="J34" s="7" t="inlineStr">
+        <is>
+          <t>scripts/check.sh run against Docker Redis+Mailpit and a local Postgres (proto-gen --check, gofmt/vet/lint, go test -cover, svelte-check, vitest coverage, real-stack Playwright e2e); FSD 3.5/5/6/8.6/10.1/11.1 updates; CLAUDE.md bullets for services/rbac and the two new frontend surfaces; this tracker</t>
+        </is>
+      </c>
+      <c r="K34" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="7" t="inlineStr">
+        <is>
           <t>Backlog: Should-have and later phases</t>
         </is>
       </c>
-      <c r="B34" s="7" t="inlineStr">
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>BL.1</t>
+        </is>
+      </c>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>Backlog: Notifications — Scheduled and transactional email/WhatsApp notifications</t>
+        </is>
+      </c>
+      <c r="D35" s="7" t="inlineStr">
+        <is>
+          <t>services/notification</t>
+        </is>
+      </c>
+      <c r="E35" s="7" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F35" s="7" t="inlineStr"/>
+      <c r="G35" s="7" t="inlineStr"/>
+      <c r="H35" s="7" t="inlineStr"/>
+      <c r="I35" s="7" t="inlineStr">
+        <is>
+          <t>FR-08.1-08.2</t>
+        </is>
+      </c>
+      <c r="J35" s="7" t="inlineStr">
+        <is>
+          <t>Event reminders, reveal notices, expiry warnings</t>
+        </is>
+      </c>
+      <c r="K35" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="7" t="inlineStr">
+        <is>
+          <t>Backlog: Should-have and later phases</t>
+        </is>
+      </c>
+      <c r="B36" s="7" t="inlineStr">
+        <is>
+          <t>BL.2</t>
+        </is>
+      </c>
+      <c r="C36" s="7" t="inlineStr">
+        <is>
+          <t>Backlog: Hall of Fame — Host-curated highlights visible to guests</t>
+        </is>
+      </c>
+      <c r="D36" s="7" t="inlineStr">
+        <is>
+          <t>services/gallery</t>
+        </is>
+      </c>
+      <c r="E36" s="7" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F36" s="7" t="inlineStr"/>
+      <c r="G36" s="7" t="inlineStr"/>
+      <c r="H36" s="7" t="inlineStr"/>
+      <c r="I36" s="7" t="inlineStr">
+        <is>
+          <t>FR-11.1-11.5</t>
+        </is>
+      </c>
+      <c r="J36" s="7" t="inlineStr">
+        <is>
+          <t>Curation, ordering and sharing of the best photos</t>
+        </is>
+      </c>
+      <c r="K36" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="7" t="inlineStr">
+        <is>
+          <t>Backlog: Should-have and later phases</t>
+        </is>
+      </c>
+      <c r="B37" s="7" t="inlineStr">
         <is>
           <t>BL.3</t>
         </is>
       </c>
-      <c r="C34" s="7" t="inlineStr">
+      <c r="C37" s="7" t="inlineStr">
         <is>
           <t>Backlog: Personal/Instant Mode (v1.1) — Capture without an event and send results to several recipients</t>
         </is>
       </c>
-      <c r="D34" s="7" t="inlineStr">
+      <c r="D37" s="7" t="inlineStr">
         <is>
           <t>apps/web, services/media</t>
         </is>
       </c>
-      <c r="E34" s="7" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F34" s="7" t="inlineStr"/>
-      <c r="G34" s="7" t="inlineStr"/>
-      <c r="H34" s="7" t="inlineStr"/>
-      <c r="I34" s="7" t="inlineStr">
+      <c r="E37" s="7" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F37" s="7" t="inlineStr"/>
+      <c r="G37" s="7" t="inlineStr"/>
+      <c r="H37" s="7" t="inlineStr"/>
+      <c r="I37" s="7" t="inlineStr">
         <is>
           <t>FR-10.1-10.7</t>
         </is>
       </c>
-      <c r="J34" s="7" t="inlineStr">
+      <c r="J37" s="7" t="inlineStr">
         <is>
           <t>Deferred until Event Mode is stable</t>
         </is>
       </c>
-      <c r="K34" s="7" t="inlineStr">
+      <c r="K37" s="7" t="inlineStr">
         <is>
           <t>2026-09-19</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K34"/>
-  <conditionalFormatting sqref="E2:E34">
+  <autoFilter ref="A1:K37"/>
+  <conditionalFormatting sqref="E2:E37">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$E2="Not Started"</formula>
     </cfRule>
@@ -2792,7 +2982,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="E2:E34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E2:E37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Not Started,In Progress,Pending Verification,Completed"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2806,7 +2996,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H23"/>
+  <dimension ref="A1:H26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3785,8 +3975,134 @@
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>Milestone 8: RBAC foundation (cross-cutting platform work)</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>apps/web</t>
+        </is>
+      </c>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>T9.2</t>
+        </is>
+      </c>
+      <c r="D24" s="7" t="inlineStr">
+        <is>
+          <t>Added the rbac API client, a best-effort profile fetch in the root layout, a dynamic Nav component, a real dark theme palette, and a new /settings page with real EN/ID language and theme switching.</t>
+        </is>
+      </c>
+      <c r="E24" s="7" t="inlineStr">
+        <is>
+          <t>The root layout's load() now returns a required profile field, which is merged into every page's PageData type (existing dashboard tests updated to pass profile: null).</t>
+        </is>
+      </c>
+      <c r="F24" s="7" t="inlineStr">
+        <is>
+          <t>Only the nav and the new settings page get real i18n; the three existing host pages keep hardcoded Indonesian text (a larger, separate retrofit). A failed/401 profile fetch resolves to profile: null rather than throwing, so /auth/login never breaks. PATCH only sets concrete theme/language values, not 'clear back to inherited' (fast-follow).</t>
+        </is>
+      </c>
+      <c r="G24" s="7" t="inlineStr">
+        <is>
+          <t>14bc5fe e1cb469 6dea65a 23963e0 d98a473 694ba26 4be3c95 99c2c86 21fbdb5</t>
+        </is>
+      </c>
+      <c r="H24" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>Milestone 8: RBAC foundation (cross-cutting platform work)</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>docs, docs/tracking</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>T9.3</t>
+        </is>
+      </c>
+      <c r="D25" s="7" t="inlineStr">
+        <is>
+          <t>Verified the RBAC foundation against the real stack (Docker Redis+Mailpit, local Postgres, scripts/check.sh) and synced the FSD, CLAUDE.md and this tracker for Task 9.</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+      <c r="F25" s="7" t="inlineStr">
+        <is>
+          <t>RBAC isn't tied to a numbered FR yet; no ID was invented (see FSD 11.1). Menu nesting and the dropdown tables are built and tested but unseeded, since no second real menu destination or dropdown consumer exists yet. Numbered this Task 9, not Task 8: the FSD (gitignored, not tracked here before now) already used 'Task 8' for a planned Milestone 2 migration (guest_sessions/media, FSD change-note v2.9→v2.10) that has no corresponding code or tracker entry yet — a pre-existing drift between the FSD and this tracker, left as discovered rather than silently reconciled. docs/ is gitignored, so these edits are not versioned in git.</t>
+        </is>
+      </c>
+      <c r="G25" s="7" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H25" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>Milestone 8: RBAC foundation (cross-cutting platform work)</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>internal/db, services/rbac, services/event, cmd/api</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>T9.1</t>
+        </is>
+      </c>
+      <c r="D26" s="7" t="inlineStr">
+        <is>
+          <t>Implemented the RBAC foundation for real: migrations for roles/menus/dropdowns/actions/permissions, a services/rbac package (Postgres repository, Service resolving per-role menus/actions/dropdowns/preferences with a host-then-role-then-global fallback chain), GET /api/v1/auth/me and PATCH /api/v1/me/preferences, and events:create enforcement on the already-shipped POST /api/v1/events.</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="inlineStr">
+        <is>
+          <t>POST /api/v1/events now requires the events:create permission in addition to a host session; every existing host is granted it by default in the seed, so behavior is unchanged unless a permission is explicitly revoked.</t>
+        </is>
+      </c>
+      <c r="F26" s="7" t="inlineStr">
+        <is>
+          <t>Fallback-chain and ancestor-inclusion logic lives in Go (table-driven tested), not PL/pgSQL, matching this codebase's zero-stored-procedure convention; the one exception is a menu cycle-prevention trigger, a genuine data-integrity invariant a CHECK can't express. Seed data stays minimal and real: 2 flat menus (events_new, settings), 2 enforced permissions (events:create, profile:update); dropdowns and nested menus are schema-complete and tested but unseeded, since no real consumer exists yet. REST only, no gRPC, for /auth/me (fast-follow, mirrors Task 5's precedent). No permission-check caching (single API instance).</t>
+        </is>
+      </c>
+      <c r="G26" s="7" t="inlineStr">
+        <is>
+          <t>85ac425 cf5f3a8 e76992d b85cbb8 08d0812 1bc1ec4 68ae150 bb79173</t>
+        </is>
+      </c>
+      <c r="H26" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H23"/>
+  <autoFilter ref="A1:H26"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
docs: record Milestone 2 Tasks 8.2 and 8.3 in the progress tracker
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/tracking/SELA_Progress_Tracker.xlsx
+++ b/docs/tracking/SELA_Progress_Tracker.xlsx
@@ -14,8 +14,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Tracker'!$A$1:$K$38</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Change Log'!$A$1:$H$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Tracker'!$A$1:$K$42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Change Log'!$A$1:$H$32</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Traceability'!$A$1:$G$59</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1013,7 +1013,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K38"/>
+  <dimension ref="A1:K42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2415,7 +2415,7 @@
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>Milestone 2 (not yet planned) — Guest scan, camera, upload with quota, gallery upload</t>
+          <t>Milestone 2: remaining guest work — Guest camera PWA (getUserMedia, post-shutter canvas, offline upload queue), event status messages and category theme (FR-02.3, FR-02.4), collage, gallery-upload toggle</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
@@ -2433,7 +2433,7 @@
       <c r="H26" s="7" t="inlineStr"/>
       <c r="I26" s="7" t="inlineStr">
         <is>
-          <t>FR-02.1-02.4, FR-03.1-03.6, FR-04.1-04.2, FR-SEC.2, FR-SEC.3</t>
+          <t>FR-02.3, FR-02.4, FR-03.1, FR-03.2, FR-03.4, FR-03.5, FR-03.6, FR-04.2</t>
         </is>
       </c>
       <c r="J26" s="7" t="inlineStr">
@@ -2443,7 +2443,7 @@
       </c>
       <c r="K26" s="7" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
@@ -2460,7 +2460,7 @@
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>Task 8: Guest session and media schema — Migration 0004 (guest_sessions, media, events.involves_minors) and the services/media domain types</t>
+          <t>Task 8: Guest session and media schema — Migration 0006 (renumbered from 0004; guest_sessions, media, events.involves_minors) and the services/media domain types</t>
         </is>
       </c>
       <c r="D27" s="7" t="inlineStr">
@@ -2470,7 +2470,7 @@
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
-          <t>Pending Verification</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="F27" s="7" t="inlineStr">
@@ -2495,7 +2495,7 @@
       </c>
       <c r="J27" s="7" t="inlineStr">
         <is>
-          <t>Schema with the same-event session key, Hall of Fame rules and gallery indexes. Open: the Go schema tests were mirrored against Postgres 16 (49/49) and type-checked, but scripts/check.sh has not run on this change yet</t>
+          <t>Schema with the same-event session key, Hall of Fame rules and gallery indexes. Verified with scripts/check.sh (full gate incl. e2e) after the renumber fix 9328b69/badcd79</t>
         </is>
       </c>
       <c r="K27" s="7" t="inlineStr">
@@ -2507,112 +2507,136 @@
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>Milestone 3: Role-correct gallery</t>
+          <t>Milestone 2: Guest captures and uploads</t>
         </is>
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>M3.1</t>
+          <t>T8.2</t>
         </is>
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>Milestone 3 (not yet planned) — Role-correct gallery, reveal timer, real-time channels</t>
+          <t>Task 8.2: Guest session and shot quota — Anonymous guest session (POST .../guest-session, sela_guest cookie), Redis session store and atomic per-session shot quota with rollback</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>services/gallery, services/realtime</t>
+          <t>services/media, internal/config</t>
         </is>
       </c>
       <c r="E28" s="7" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F28" s="7" t="inlineStr"/>
-      <c r="G28" s="7" t="inlineStr"/>
-      <c r="H28" s="7" t="inlineStr"/>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F28" s="7" t="inlineStr">
+        <is>
+          <t>83213fa 69a73cb</t>
+        </is>
+      </c>
+      <c r="G28" s="7" t="inlineStr">
+        <is>
+          <t>92f231d 4bb836c</t>
+        </is>
+      </c>
+      <c r="H28" s="7" t="inlineStr">
+        <is>
+          <t>83.1% (services/media), 100% (internal/config)</t>
+        </is>
+      </c>
       <c r="I28" s="7" t="inlineStr">
         <is>
-          <t>FR-05.1-05.6</t>
+          <t>FR-02.1, FR-02.2, FR-03.3</t>
         </is>
       </c>
       <c r="J28" s="7" t="inlineStr">
         <is>
-          <t>Host sees all media, guest only their own, WebSocket channels split by role</t>
+          <t>Session create/resume for active events only; token hashed in Redis (guest:*) with GUEST_SESSION_TTL; Lua reserve/release on quota:{event}:{session} seeded from media rows; 20-way concurrency test never overspends. scripts/check.sh passed (proto, gofmt, vet, lint, Go + web tests, e2e 10/10)</t>
         </is>
       </c>
       <c r="K28" s="7" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
         <is>
-          <t>Milestone 4: Moderate and export</t>
+          <t>Milestone 2: Guest captures and uploads</t>
         </is>
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>M4.1</t>
+          <t>T8.3</t>
         </is>
       </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>Milestone 4 (not yet planned) — Moderation and full-gallery ZIP export</t>
+          <t>Task 8.3: Direct upload, processing and gallery visibility — S3 object store (MinIO dev bucket), pre-signed PUT for exact size/type, magic-byte check and EXIF/GPS stripping, sweeper, my-media / hall-of-fame / host media endpoints with SQL-level visibility</t>
         </is>
       </c>
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>services/gallery, services/media</t>
+          <t>internal/objstore, services/media, services/media/strip, cmd/api, deploy</t>
         </is>
       </c>
       <c r="E29" s="7" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F29" s="7" t="inlineStr"/>
-      <c r="G29" s="7" t="inlineStr"/>
-      <c r="H29" s="7" t="inlineStr"/>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F29" s="7" t="inlineStr">
+        <is>
+          <t>459695b 4263b3d 69a73cb d8a0998 ac399ad</t>
+        </is>
+      </c>
+      <c r="G29" s="7" t="inlineStr">
+        <is>
+          <t>82f84fd 3bfd703 4bb836c 22eb226 b08dd6a b2cd6b2</t>
+        </is>
+      </c>
+      <c r="H29" s="7" t="inlineStr">
+        <is>
+          <t>83.1% (services/media), 82.3% (strip), 90.4% (internal/objstore), 82.8% (cmd/api)</t>
+        </is>
+      </c>
       <c r="I29" s="7" t="inlineStr">
         <is>
-          <t>FR-06.1-06.4, FR-07.1-07.3</t>
+          <t>FR-04.1, FR-05.5, FR-05.6, FR-SEC.1, FR-SEC.2, FR-SEC.3, FR-SEC.10</t>
         </is>
       </c>
       <c r="J29" s="7" t="inlineStr">
         <is>
-          <t>Hide/delete, asynchronous ZIP export, share links</t>
+          <t>JPEG/PNG/WebP up to 20 MB; HEIC and video refused (415) until they can be stripped. Smoke-tested against the real API, Redis and MinIO: signed PUT 200, wrong type 403, served photo has no EXIF/GPS, quota 429, guest isolation, no-cookie 401. scripts/check.sh passed (proto, gofmt, vet, lint, Go + web tests, e2e 10/10)</t>
         </is>
       </c>
       <c r="K29" s="7" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
         <is>
-          <t>Milestone 5: Plans and payment</t>
+          <t>Milestone 2: Guest captures and uploads</t>
         </is>
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>M5.1</t>
+          <t>T8.4</t>
         </is>
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>Milestone 5 (not yet planned) — Plans, package recommendation and payment (QRIS, e-wallet, card)</t>
+          <t>HEIC and video metadata stripping — Choose and add a metadata-rewriting tool for HEIC and MP4/MOV, then accept those types (video limit 200 MB)</t>
         </is>
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>services/payment, services/event</t>
+          <t>services/media</t>
         </is>
       </c>
       <c r="E30" s="7" t="inlineStr">
@@ -2625,39 +2649,39 @@
       <c r="H30" s="7" t="inlineStr"/>
       <c r="I30" s="7" t="inlineStr">
         <is>
-          <t>FR-01.5, FR-01.6, FR-09.2, FR-09.3</t>
+          <t>FR-04.1, FR-SEC.2</t>
         </is>
       </c>
       <c r="J30" s="7" t="inlineStr">
         <is>
-          <t>Free and paid tiers by event scale; micro-payments; transaction history</t>
+          <t>Follow-up from T8.3</t>
         </is>
       </c>
       <c r="K30" s="7" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
         <is>
-          <t>Milestone 6: Privacy and compliance readiness</t>
+          <t>Milestone 2: Guest captures and uploads</t>
         </is>
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>M6.1</t>
+          <t>T8.5</t>
         </is>
       </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
-          <t>Milestone 6 (not yet planned) — Privacy and compliance readiness</t>
+          <t>Guest upload and session rate limits — Redis rate limits on guest-session creation and uploads (per session and per connection address)</t>
         </is>
       </c>
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>cross-cutting</t>
+          <t>services/media</t>
         </is>
       </c>
       <c r="E31" s="7" t="inlineStr">
@@ -2670,39 +2694,39 @@
       <c r="H31" s="7" t="inlineStr"/>
       <c r="I31" s="7" t="inlineStr">
         <is>
-          <t>FR-SEC.1, FR-SEC.5-SEC.8, FR-SEC.10</t>
+          <t>FR-SEC.9</t>
         </is>
       </c>
       <c r="J31" s="7" t="inlineStr">
         <is>
-          <t>PII column encryption with a blind index, audit log, retention and deletion, child-event defaults, noindex headers</t>
+          <t>Follow-up from T8.2/T8.3</t>
         </is>
       </c>
       <c r="K31" s="7" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
         <is>
-          <t>Milestone 7: Closed beta</t>
+          <t>Milestone 3: Role-correct gallery</t>
         </is>
       </c>
       <c r="B32" s="7" t="inlineStr">
         <is>
-          <t>M7.1</t>
+          <t>M3.1</t>
         </is>
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>Milestone 7 (not yet planned) — Closed beta across wedding, graduation and birthday events</t>
+          <t>Milestone 3 (not yet planned) — Role-correct gallery, reveal timer, real-time channels</t>
         </is>
       </c>
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>operations</t>
+          <t>services/gallery, services/realtime</t>
         </is>
       </c>
       <c r="E32" s="7" t="inlineStr">
@@ -2713,10 +2737,14 @@
       <c r="F32" s="7" t="inlineStr"/>
       <c r="G32" s="7" t="inlineStr"/>
       <c r="H32" s="7" t="inlineStr"/>
-      <c r="I32" s="7" t="inlineStr"/>
+      <c r="I32" s="7" t="inlineStr">
+        <is>
+          <t>FR-05.1-05.6</t>
+        </is>
+      </c>
       <c r="J32" s="7" t="inlineStr">
         <is>
-          <t>Validate the hypothesis and fill the TBD success metrics in the PRD</t>
+          <t>Host sees all media, guest only their own, WebSocket channels split by role</t>
         </is>
       </c>
       <c r="K32" s="7" t="inlineStr">
@@ -2728,181 +2756,157 @@
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
         <is>
-          <t>Milestone 8: RBAC foundation (cross-cutting platform work)</t>
+          <t>Milestone 4: Moderate and export</t>
         </is>
       </c>
       <c r="B33" s="7" t="inlineStr">
         <is>
-          <t>T9.1</t>
+          <t>M4.1</t>
         </is>
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>Task 9: RBAC foundation — RBAC schema (roles, menus, dropdowns, actions/permissions) and the services/rbac backend package; events:create gated on the already-shipped create-event route</t>
+          <t>Milestone 4 (not yet planned) — Moderation and full-gallery ZIP export</t>
         </is>
       </c>
       <c r="D33" s="7" t="inlineStr">
         <is>
-          <t>internal/db (0004, 0005), services/rbac, services/event, cmd/api</t>
+          <t>services/gallery, services/media</t>
         </is>
       </c>
       <c r="E33" s="7" t="inlineStr">
         <is>
-          <t>Completed</t>
-        </is>
-      </c>
-      <c r="F33" s="7" t="inlineStr">
-        <is>
-          <t>85ac425 e76992d 08d0812 68ae150</t>
-        </is>
-      </c>
-      <c r="G33" s="7" t="inlineStr">
-        <is>
-          <t>cf5f3a8 b85cbb8 1bc1ec4 bb79173</t>
-        </is>
-      </c>
-      <c r="H33" s="7" t="inlineStr">
-        <is>
-          <t>services/rbac 81.9%; services/event 91.3%; cmd/api 83.3%</t>
-        </is>
-      </c>
-      <c r="I33" s="7" t="inlineStr"/>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F33" s="7" t="inlineStr"/>
+      <c r="G33" s="7" t="inlineStr"/>
+      <c r="H33" s="7" t="inlineStr"/>
+      <c r="I33" s="7" t="inlineStr">
+        <is>
+          <t>FR-06.1-06.4, FR-07.1-07.3</t>
+        </is>
+      </c>
       <c r="J33" s="7" t="inlineStr">
         <is>
-          <t>migrations 0004_rbac_foundation.sql, 0005_hosts_role_and_preferences.sql; services/rbac (types/postgres/service/http) with GET /api/v1/auth/me and PATCH /api/v1/me/preferences; RequirePermission wired onto POST /api/v1/events (events:create); seed limited to 2 menus (events_new, settings) and 2 enforced permissions (events:create, profile:update), every existing host granted both so no current behavior changes</t>
+          <t>Hide/delete, asynchronous ZIP export, share links</t>
         </is>
       </c>
       <c r="K33" s="7" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-19</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
         <is>
-          <t>Milestone 8: RBAC foundation (cross-cutting platform work)</t>
+          <t>Milestone 5: Plans and payment</t>
         </is>
       </c>
       <c r="B34" s="7" t="inlineStr">
         <is>
-          <t>T9.2</t>
+          <t>M5.1</t>
         </is>
       </c>
       <c r="C34" s="7" t="inlineStr">
         <is>
-          <t>Task 9: RBAC foundation — Frontend: rbac API client, best-effort profile fetch in the root layout, dynamic Nav, dark theme palette, and the new /settings page with real EN/ID switching</t>
+          <t>Milestone 5 (not yet planned) — Plans, package recommendation and payment (QRIS, e-wallet, card)</t>
         </is>
       </c>
       <c r="D34" s="7" t="inlineStr">
         <is>
-          <t>apps/web</t>
+          <t>services/payment, services/event</t>
         </is>
       </c>
       <c r="E34" s="7" t="inlineStr">
         <is>
-          <t>Completed</t>
-        </is>
-      </c>
-      <c r="F34" s="7" t="inlineStr">
-        <is>
-          <t>14bc5fe 6dea65a 4be3c95</t>
-        </is>
-      </c>
-      <c r="G34" s="7" t="inlineStr">
-        <is>
-          <t>21fbdb5 e1cb469 23963e0 d98a473 694ba26 99c2c86</t>
-        </is>
-      </c>
-      <c r="H34" s="7" t="inlineStr">
-        <is>
-          <t>184 tests pass; 97.16% statements / 89.65% branches / 97.6% functions / 99.75% lines; svelte-check 0 errors/0 warnings</t>
-        </is>
-      </c>
-      <c r="I34" s="7" t="inlineStr"/>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F34" s="7" t="inlineStr"/>
+      <c r="G34" s="7" t="inlineStr"/>
+      <c r="H34" s="7" t="inlineStr"/>
+      <c r="I34" s="7" t="inlineStr">
+        <is>
+          <t>FR-01.5, FR-01.6, FR-09.2, FR-09.3</t>
+        </is>
+      </c>
       <c r="J34" s="7" t="inlineStr">
         <is>
-          <t>src/lib/api/rbac.ts; src/lib/components/Nav.svelte; :root[data-theme='dark'] palette in tokens.css; +layout.ts best-effort getProfile() (swallows a 401 so /auth/login never breaks); +layout.svelte renders Nav and sets document.documentElement.dataset.theme; src/routes/settings/+page.svelte (role, theme toggle, language toggle, own local EN/ID string table); the three pre-existing host pages keep their hardcoded Indonesian text unchanged</t>
+          <t>Free and paid tiers by event scale; micro-payments; transaction history</t>
         </is>
       </c>
       <c r="K34" s="7" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-19</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
         <is>
-          <t>Milestone 8: RBAC foundation (cross-cutting platform work)</t>
+          <t>Milestone 6: Privacy and compliance readiness</t>
         </is>
       </c>
       <c r="B35" s="7" t="inlineStr">
         <is>
-          <t>T9.3</t>
+          <t>M6.1</t>
         </is>
       </c>
       <c r="C35" s="7" t="inlineStr">
         <is>
-          <t>Task 9: RBAC foundation — Real-stack verification and docs/tracking sync for Task 8</t>
+          <t>Milestone 6 (not yet planned) — Privacy and compliance readiness</t>
         </is>
       </c>
       <c r="D35" s="7" t="inlineStr">
         <is>
-          <t>docs, docs/tracking, CLAUDE.md</t>
+          <t>cross-cutting</t>
         </is>
       </c>
       <c r="E35" s="7" t="inlineStr">
         <is>
-          <t>Completed</t>
-        </is>
-      </c>
-      <c r="F35" s="7" t="inlineStr">
-        <is>
-          <t>n/a (documentation)</t>
-        </is>
-      </c>
-      <c r="G35" s="7" t="inlineStr">
-        <is>
-          <t>n/a (docs/ is gitignored, not committed)</t>
-        </is>
-      </c>
-      <c r="H35" s="7" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="I35" s="7" t="inlineStr"/>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F35" s="7" t="inlineStr"/>
+      <c r="G35" s="7" t="inlineStr"/>
+      <c r="H35" s="7" t="inlineStr"/>
+      <c r="I35" s="7" t="inlineStr">
+        <is>
+          <t>FR-SEC.1, FR-SEC.5-SEC.8, FR-SEC.10</t>
+        </is>
+      </c>
       <c r="J35" s="7" t="inlineStr">
         <is>
-          <t>scripts/check.sh run against Docker Redis+Mailpit and a local Postgres (proto-gen --check, gofmt/vet/lint, go test -cover, svelte-check, vitest coverage, real-stack Playwright e2e); FSD 3.5/5/6/8.6/10.1/11.1 updates; CLAUDE.md bullets for services/rbac and the two new frontend surfaces; this tracker</t>
+          <t>PII column encryption with a blind index, audit log, retention and deletion, child-event defaults, noindex headers</t>
         </is>
       </c>
       <c r="K35" s="7" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-19</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
         <is>
-          <t>Backlog: Should-have and later phases</t>
+          <t>Milestone 7: Closed beta</t>
         </is>
       </c>
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t>BL.1</t>
+          <t>M7.1</t>
         </is>
       </c>
       <c r="C36" s="7" t="inlineStr">
         <is>
-          <t>Backlog: Notifications — Scheduled and transactional email/WhatsApp notifications</t>
+          <t>Milestone 7 (not yet planned) — Closed beta across wedding, graduation and birthday events</t>
         </is>
       </c>
       <c r="D36" s="7" t="inlineStr">
         <is>
-          <t>services/notification</t>
+          <t>operations</t>
         </is>
       </c>
       <c r="E36" s="7" t="inlineStr">
@@ -2913,14 +2917,10 @@
       <c r="F36" s="7" t="inlineStr"/>
       <c r="G36" s="7" t="inlineStr"/>
       <c r="H36" s="7" t="inlineStr"/>
-      <c r="I36" s="7" t="inlineStr">
-        <is>
-          <t>FR-08.1-08.2</t>
-        </is>
-      </c>
+      <c r="I36" s="7" t="inlineStr"/>
       <c r="J36" s="7" t="inlineStr">
         <is>
-          <t>Event reminders, reveal notices, expiry warnings</t>
+          <t>Validate the hypothesis and fill the TBD success metrics in the PRD</t>
         </is>
       </c>
       <c r="K36" s="7" t="inlineStr">
@@ -2932,96 +2932,300 @@
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
         <is>
-          <t>Backlog: Should-have and later phases</t>
+          <t>Milestone 8: RBAC foundation (cross-cutting platform work)</t>
         </is>
       </c>
       <c r="B37" s="7" t="inlineStr">
         <is>
-          <t>BL.2</t>
+          <t>T9.1</t>
         </is>
       </c>
       <c r="C37" s="7" t="inlineStr">
         <is>
-          <t>Backlog: Hall of Fame — Host-curated highlights visible to guests</t>
+          <t>Task 9: RBAC foundation — RBAC schema (roles, menus, dropdowns, actions/permissions) and the services/rbac backend package; events:create gated on the already-shipped create-event route</t>
         </is>
       </c>
       <c r="D37" s="7" t="inlineStr">
         <is>
-          <t>services/gallery</t>
+          <t>internal/db (0004, 0005), services/rbac, services/event, cmd/api</t>
         </is>
       </c>
       <c r="E37" s="7" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F37" s="7" t="inlineStr"/>
-      <c r="G37" s="7" t="inlineStr"/>
-      <c r="H37" s="7" t="inlineStr"/>
-      <c r="I37" s="7" t="inlineStr">
-        <is>
-          <t>FR-11.1-11.5</t>
-        </is>
-      </c>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F37" s="7" t="inlineStr">
+        <is>
+          <t>85ac425 e76992d 08d0812 68ae150</t>
+        </is>
+      </c>
+      <c r="G37" s="7" t="inlineStr">
+        <is>
+          <t>cf5f3a8 b85cbb8 1bc1ec4 bb79173</t>
+        </is>
+      </c>
+      <c r="H37" s="7" t="inlineStr">
+        <is>
+          <t>services/rbac 81.9%; services/event 91.3%; cmd/api 83.3%</t>
+        </is>
+      </c>
+      <c r="I37" s="7" t="inlineStr"/>
       <c r="J37" s="7" t="inlineStr">
         <is>
-          <t>Curation, ordering and sharing of the best photos</t>
+          <t>migrations 0004_rbac_foundation.sql, 0005_hosts_role_and_preferences.sql; services/rbac (types/postgres/service/http) with GET /api/v1/auth/me and PATCH /api/v1/me/preferences; RequirePermission wired onto POST /api/v1/events (events:create); seed limited to 2 menus (events_new, settings) and 2 enforced permissions (events:create, profile:update), every existing host granted both so no current behavior changes</t>
         </is>
       </c>
       <c r="K37" s="7" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
         <is>
+          <t>Milestone 8: RBAC foundation (cross-cutting platform work)</t>
+        </is>
+      </c>
+      <c r="B38" s="7" t="inlineStr">
+        <is>
+          <t>T9.2</t>
+        </is>
+      </c>
+      <c r="C38" s="7" t="inlineStr">
+        <is>
+          <t>Task 9: RBAC foundation — Frontend: rbac API client, best-effort profile fetch in the root layout, dynamic Nav, dark theme palette, and the new /settings page with real EN/ID switching</t>
+        </is>
+      </c>
+      <c r="D38" s="7" t="inlineStr">
+        <is>
+          <t>apps/web</t>
+        </is>
+      </c>
+      <c r="E38" s="7" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F38" s="7" t="inlineStr">
+        <is>
+          <t>14bc5fe 6dea65a 4be3c95</t>
+        </is>
+      </c>
+      <c r="G38" s="7" t="inlineStr">
+        <is>
+          <t>21fbdb5 e1cb469 23963e0 d98a473 694ba26 99c2c86</t>
+        </is>
+      </c>
+      <c r="H38" s="7" t="inlineStr">
+        <is>
+          <t>184 tests pass; 97.16% statements / 89.65% branches / 97.6% functions / 99.75% lines; svelte-check 0 errors/0 warnings</t>
+        </is>
+      </c>
+      <c r="I38" s="7" t="inlineStr"/>
+      <c r="J38" s="7" t="inlineStr">
+        <is>
+          <t>src/lib/api/rbac.ts; src/lib/components/Nav.svelte; :root[data-theme='dark'] palette in tokens.css; +layout.ts best-effort getProfile() (swallows a 401 so /auth/login never breaks); +layout.svelte renders Nav and sets document.documentElement.dataset.theme; src/routes/settings/+page.svelte (role, theme toggle, language toggle, own local EN/ID string table); the three pre-existing host pages keep their hardcoded Indonesian text unchanged</t>
+        </is>
+      </c>
+      <c r="K38" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="7" t="inlineStr">
+        <is>
+          <t>Milestone 8: RBAC foundation (cross-cutting platform work)</t>
+        </is>
+      </c>
+      <c r="B39" s="7" t="inlineStr">
+        <is>
+          <t>T9.3</t>
+        </is>
+      </c>
+      <c r="C39" s="7" t="inlineStr">
+        <is>
+          <t>Task 9: RBAC foundation — Real-stack verification and docs/tracking sync for Task 8</t>
+        </is>
+      </c>
+      <c r="D39" s="7" t="inlineStr">
+        <is>
+          <t>docs, docs/tracking, CLAUDE.md</t>
+        </is>
+      </c>
+      <c r="E39" s="7" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F39" s="7" t="inlineStr">
+        <is>
+          <t>n/a (documentation)</t>
+        </is>
+      </c>
+      <c r="G39" s="7" t="inlineStr">
+        <is>
+          <t>n/a (docs/ is gitignored, not committed)</t>
+        </is>
+      </c>
+      <c r="H39" s="7" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I39" s="7" t="inlineStr"/>
+      <c r="J39" s="7" t="inlineStr">
+        <is>
+          <t>scripts/check.sh run against Docker Redis+Mailpit and a local Postgres (proto-gen --check, gofmt/vet/lint, go test -cover, svelte-check, vitest coverage, real-stack Playwright e2e); FSD 3.5/5/6/8.6/10.1/11.1 updates; CLAUDE.md bullets for services/rbac and the two new frontend surfaces; this tracker</t>
+        </is>
+      </c>
+      <c r="K39" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="7" t="inlineStr">
+        <is>
           <t>Backlog: Should-have and later phases</t>
         </is>
       </c>
-      <c r="B38" s="7" t="inlineStr">
+      <c r="B40" s="7" t="inlineStr">
+        <is>
+          <t>BL.1</t>
+        </is>
+      </c>
+      <c r="C40" s="7" t="inlineStr">
+        <is>
+          <t>Backlog: Notifications — Scheduled and transactional email/WhatsApp notifications</t>
+        </is>
+      </c>
+      <c r="D40" s="7" t="inlineStr">
+        <is>
+          <t>services/notification</t>
+        </is>
+      </c>
+      <c r="E40" s="7" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F40" s="7" t="inlineStr"/>
+      <c r="G40" s="7" t="inlineStr"/>
+      <c r="H40" s="7" t="inlineStr"/>
+      <c r="I40" s="7" t="inlineStr">
+        <is>
+          <t>FR-08.1-08.2</t>
+        </is>
+      </c>
+      <c r="J40" s="7" t="inlineStr">
+        <is>
+          <t>Event reminders, reveal notices, expiry warnings</t>
+        </is>
+      </c>
+      <c r="K40" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="7" t="inlineStr">
+        <is>
+          <t>Backlog: Should-have and later phases</t>
+        </is>
+      </c>
+      <c r="B41" s="7" t="inlineStr">
+        <is>
+          <t>BL.2</t>
+        </is>
+      </c>
+      <c r="C41" s="7" t="inlineStr">
+        <is>
+          <t>Backlog: Hall of Fame — Host-curated highlights visible to guests</t>
+        </is>
+      </c>
+      <c r="D41" s="7" t="inlineStr">
+        <is>
+          <t>services/gallery</t>
+        </is>
+      </c>
+      <c r="E41" s="7" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F41" s="7" t="inlineStr"/>
+      <c r="G41" s="7" t="inlineStr"/>
+      <c r="H41" s="7" t="inlineStr"/>
+      <c r="I41" s="7" t="inlineStr">
+        <is>
+          <t>FR-11.1-11.5</t>
+        </is>
+      </c>
+      <c r="J41" s="7" t="inlineStr">
+        <is>
+          <t>Curation, ordering and sharing of the best photos</t>
+        </is>
+      </c>
+      <c r="K41" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="7" t="inlineStr">
+        <is>
+          <t>Backlog: Should-have and later phases</t>
+        </is>
+      </c>
+      <c r="B42" s="7" t="inlineStr">
         <is>
           <t>BL.3</t>
         </is>
       </c>
-      <c r="C38" s="7" t="inlineStr">
+      <c r="C42" s="7" t="inlineStr">
         <is>
           <t>Backlog: Personal/Instant Mode (v1.1) — Capture without an event and send results to several recipients</t>
         </is>
       </c>
-      <c r="D38" s="7" t="inlineStr">
+      <c r="D42" s="7" t="inlineStr">
         <is>
           <t>apps/web, services/media</t>
         </is>
       </c>
-      <c r="E38" s="7" t="inlineStr">
+      <c r="E42" s="7" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="F38" s="7" t="inlineStr"/>
-      <c r="G38" s="7" t="inlineStr"/>
-      <c r="H38" s="7" t="inlineStr"/>
-      <c r="I38" s="7" t="inlineStr">
+      <c r="F42" s="7" t="inlineStr"/>
+      <c r="G42" s="7" t="inlineStr"/>
+      <c r="H42" s="7" t="inlineStr"/>
+      <c r="I42" s="7" t="inlineStr">
         <is>
           <t>FR-10.1-10.7</t>
         </is>
       </c>
-      <c r="J38" s="7" t="inlineStr">
+      <c r="J42" s="7" t="inlineStr">
         <is>
           <t>Deferred until Event Mode is stable</t>
         </is>
       </c>
-      <c r="K38" s="7" t="inlineStr">
+      <c r="K42" s="7" t="inlineStr">
         <is>
           <t>2026-09-19</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K38"/>
-  <conditionalFormatting sqref="E2:E38">
+  <autoFilter ref="A1:K42"/>
+  <conditionalFormatting sqref="E2:E42">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$E2="Not Started"</formula>
     </cfRule>
@@ -3039,7 +3243,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="E2:E38" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E2:E42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Not Started,In Progress,Pending Verification,Completed"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3053,7 +3257,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H28"/>
+  <dimension ref="A1:H32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -4082,32 +4286,32 @@
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>internal/db, services/media</t>
+          <t>docs</t>
         </is>
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>T8.1</t>
+          <t>T8.3</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>Added migration 0004: guest_sessions, media and events.involves_minors, with schema tests and the media domain types.</t>
+          <t>Updated the FSD to v2.13 (2.4, 5, 6, 8.5-8.7, 11.1) and this tracker; added follow-ups T8.4 (HEIC/video stripping) and T8.5 (guest rate limits).</t>
         </is>
       </c>
       <c r="E25" s="7" t="inlineStr">
         <is>
-          <t>New migration 0004 (additive). events gains involves_minors boolean NOT NULL DEFAULT false.</t>
+          <t>None.</t>
         </is>
       </c>
       <c r="F25" s="7" t="inlineStr">
         <is>
-          <t>No sisa_jepretan column (Redis holds the live counter; the durable count comes from media rows). No browser fingerprint (FSD 8.11 data minimisation). processing_state is separate from the moderation status. The composite key media.(event_id, session_id) -&gt; guest_sessions keeps a session inside its own event. RESTRICT deletes, so the retention job removes stored objects first. WebP accepted beside the FR-04.1 formats because the camera pipeline outputs it (FSD 7).</t>
+          <t>FR-02.2 marked Completed at the API level; the rest stay Partial until the PWA and M3 gallery UI exist.</t>
         </is>
       </c>
       <c r="G25" s="7" t="inlineStr">
         <is>
-          <t>6d1e157 720b11f</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="H25" s="7" t="inlineStr">
@@ -4119,37 +4323,37 @@
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
         <is>
-          <t>Milestone 8: RBAC foundation (cross-cutting platform work)</t>
+          <t>Milestone 2: Guest captures and uploads</t>
         </is>
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>apps/web</t>
+          <t>internal/db, services/media</t>
         </is>
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>T9.2</t>
+          <t>T8.1</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>Added the rbac API client, a best-effort profile fetch in the root layout, a dynamic Nav component, a real dark theme palette, and a new /settings page with real EN/ID language and theme switching.</t>
+          <t>Added migration 0004: guest_sessions, media and events.involves_minors, with schema tests and the media domain types.</t>
         </is>
       </c>
       <c r="E26" s="7" t="inlineStr">
         <is>
-          <t>The root layout's load() now returns a required profile field, which is merged into every page's PageData type (existing dashboard tests updated to pass profile: null).</t>
+          <t>New migration 0004 (additive). events gains involves_minors boolean NOT NULL DEFAULT false.</t>
         </is>
       </c>
       <c r="F26" s="7" t="inlineStr">
         <is>
-          <t>Only the nav and the new settings page get real i18n; the three existing host pages keep hardcoded Indonesian text (a larger, separate retrofit). A failed/401 profile fetch resolves to profile: null rather than throwing, so /auth/login never breaks. PATCH only sets concrete theme/language values, not 'clear back to inherited' (fast-follow).</t>
+          <t>No sisa_jepretan column (Redis holds the live counter; the durable count comes from media rows). No browser fingerprint (FSD 8.11 data minimisation). processing_state is separate from the moderation status. The composite key media.(event_id, session_id) -&gt; guest_sessions keeps a session inside its own event. RESTRICT deletes, so the retention job removes stored objects first. WebP accepted beside the FR-04.1 formats because the camera pipeline outputs it (FSD 7).</t>
         </is>
       </c>
       <c r="G26" s="7" t="inlineStr">
         <is>
-          <t>14bc5fe e1cb469 6dea65a 23963e0 d98a473 694ba26 4be3c95 99c2c86 21fbdb5</t>
+          <t>6d1e157 720b11f</t>
         </is>
       </c>
       <c r="H26" s="7" t="inlineStr">
@@ -4161,37 +4365,37 @@
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
         <is>
-          <t>Milestone 8: RBAC foundation (cross-cutting platform work)</t>
+          <t>Milestone 2: Guest captures and uploads</t>
         </is>
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>docs, docs/tracking</t>
+          <t>internal/db, services/media</t>
         </is>
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>T9.3</t>
+          <t>T8.1</t>
         </is>
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>Verified the RBAC foundation against the real stack (Docker Redis+Mailpit, local Postgres, scripts/check.sh) and synced the FSD, CLAUDE.md and this tracker for Task 9.</t>
+          <t>Renumbered the guest_sessions/media migration from 0004 to 0006 so it runs after the RBAC migrations 0004/0005; added a test that migration versions are unique and that guest media runs after RBAC.</t>
         </is>
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
-          <t>None.</t>
+          <t>Migration file renamed 0004_guest_sessions_media.sql -&gt; 0006_guest_sessions_media.sql (SQL unchanged). Local databases that applied feat/guest-media alone must be recreated.</t>
         </is>
       </c>
       <c r="F27" s="7" t="inlineStr">
         <is>
-          <t>RBAC isn't tied to a numbered FR yet; no ID was invented (see FSD 11.1). Menu nesting and the dropdown tables are built and tested but unseeded, since no second real menu destination or dropdown consumer exists yet. Numbered this Task 9, not Task 8: the FSD (gitignored, not tracked here before now) already used 'Task 8' for a planned Milestone 2 migration (guest_sessions/media, FSD change-note v2.9→v2.10) that has no corresponding code or tracker entry yet — a pre-existing drift between the FSD and this tracker, left as discovered rather than silently reconciled. docs/ is gitignored, so these edits are not versioned in git.</t>
+          <t>Merging feat/guest-media and feat/rbac-foundation into development left two version-0004 files, which goose rejects. Guest media depends only on events (0003), so it moves last. Guest visibility stays as FSD 3.2/4.5 define it. FSD bumped to v2.12.</t>
         </is>
       </c>
       <c r="G27" s="7" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>9328b69 badcd79</t>
         </is>
       </c>
       <c r="H27" s="7" t="inlineStr">
@@ -4203,47 +4407,215 @@
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
         <is>
+          <t>Milestone 2: Guest captures and uploads</t>
+        </is>
+      </c>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>internal/objstore, services/media, services/media/strip, cmd/api, deploy, scripts</t>
+        </is>
+      </c>
+      <c r="C28" s="7" t="inlineStr">
+        <is>
+          <t>T8.3</t>
+        </is>
+      </c>
+      <c r="D28" s="7" t="inlineStr">
+        <is>
+          <t>Added the S3 object store with a MinIO dev bucket, direct browser uploads via pre-signed PUT, magic-byte validation and metadata stripping, an upload sweeper, and the my-media, hall-of-fame and host media endpoints with visibility enforced in SQL.</t>
+        </is>
+      </c>
+      <c r="E28" s="7" t="inlineStr">
+        <is>
+          <t>New required settings S3_ENDPOINT, S3_REGION, S3_BUCKET, S3_ACCESS_KEY_ID, S3_SECRET_ACCESS_KEY (S3_PATH_STYLE optional). deploy/docker-compose.yml adds minio and minio-init (quay.io images; needs MINIO_ROOT_USER/PASSWORD). check.sh and e2e.sh require MinIO. New deps aws-sdk-go-v2 and golang.org/x/image v0.45.0 (last release on Go 1.25).</t>
+        </is>
+      </c>
+      <c r="F28" s="7" t="inlineStr">
+        <is>
+          <t>Guest visibility stays FSD 3.2: own media only, plus the host-curated Hall of Fame after reveal; the brief's 'revealed = all media' rule was not adopted. Photos only (JPEG/PNG/WebP, 20 MB); HEIC and video are refused rather than stored unstripped. Stripping uses allow-lists and must be idempotent. noindex is sent for every event, not only children's events. The upload endpoint is split into uploads + complete instead of FSD 6's single POST .../media.</t>
+        </is>
+      </c>
+      <c r="G28" s="7" t="inlineStr">
+        <is>
+          <t>459695b 82f84fd 4263b3d 3bfd703 d8a0998 22eb226 ac399ad b08dd6a</t>
+        </is>
+      </c>
+      <c r="H28" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>Milestone 2: Guest captures and uploads</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>services/media, internal/config</t>
+        </is>
+      </c>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>T8.2</t>
+        </is>
+      </c>
+      <c r="D29" s="7" t="inlineStr">
+        <is>
+          <t>Added anonymous guest sessions (POST /api/v1/events/{event_id}/guest-session, sela_guest cookie scoped to the event's API path) and an atomic Redis shot quota with rollback.</t>
+        </is>
+      </c>
+      <c r="E29" s="7" t="inlineStr">
+        <is>
+          <t>New optional setting GUEST_SESSION_TTL (default 72h). New Redis keys guest:* and quota:*.</t>
+        </is>
+      </c>
+      <c r="F29" s="7" t="inlineStr">
+        <is>
+          <t>Session creation is a POST per FSD 6, not a side effect of GET /e/{short_code}, so link previews and crawlers create nothing. The cookie Path is /api/v1/events/{event_id} because a /e/ path would never reach the API. The quota counter reseeds from media rows, which stay the source of truth. Guest tokens reuse OTP_HMAC_KEY under their own domain prefix. The 72h TTL is a configurable default; the docs define none.</t>
+        </is>
+      </c>
+      <c r="G29" s="7" t="inlineStr">
+        <is>
+          <t>83213fa 92f231d 69a73cb 4bb836c</t>
+        </is>
+      </c>
+      <c r="H29" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="7" t="inlineStr">
+        <is>
           <t>Milestone 8: RBAC foundation (cross-cutting platform work)</t>
         </is>
       </c>
-      <c r="B28" s="7" t="inlineStr">
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>apps/web</t>
+        </is>
+      </c>
+      <c r="C30" s="7" t="inlineStr">
+        <is>
+          <t>T9.2</t>
+        </is>
+      </c>
+      <c r="D30" s="7" t="inlineStr">
+        <is>
+          <t>Added the rbac API client, a best-effort profile fetch in the root layout, a dynamic Nav component, a real dark theme palette, and a new /settings page with real EN/ID language and theme switching.</t>
+        </is>
+      </c>
+      <c r="E30" s="7" t="inlineStr">
+        <is>
+          <t>The root layout's load() now returns a required profile field, which is merged into every page's PageData type (existing dashboard tests updated to pass profile: null).</t>
+        </is>
+      </c>
+      <c r="F30" s="7" t="inlineStr">
+        <is>
+          <t>Only the nav and the new settings page get real i18n; the three existing host pages keep hardcoded Indonesian text (a larger, separate retrofit). A failed/401 profile fetch resolves to profile: null rather than throwing, so /auth/login never breaks. PATCH only sets concrete theme/language values, not 'clear back to inherited' (fast-follow).</t>
+        </is>
+      </c>
+      <c r="G30" s="7" t="inlineStr">
+        <is>
+          <t>14bc5fe e1cb469 6dea65a 23963e0 d98a473 694ba26 4be3c95 99c2c86 21fbdb5</t>
+        </is>
+      </c>
+      <c r="H30" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
+          <t>Milestone 8: RBAC foundation (cross-cutting platform work)</t>
+        </is>
+      </c>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>docs, docs/tracking</t>
+        </is>
+      </c>
+      <c r="C31" s="7" t="inlineStr">
+        <is>
+          <t>T9.3</t>
+        </is>
+      </c>
+      <c r="D31" s="7" t="inlineStr">
+        <is>
+          <t>Verified the RBAC foundation against the real stack (Docker Redis+Mailpit, local Postgres, scripts/check.sh) and synced the FSD, CLAUDE.md and this tracker for Task 9.</t>
+        </is>
+      </c>
+      <c r="E31" s="7" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+      <c r="F31" s="7" t="inlineStr">
+        <is>
+          <t>RBAC isn't tied to a numbered FR yet; no ID was invented (see FSD 11.1). Menu nesting and the dropdown tables are built and tested but unseeded, since no second real menu destination or dropdown consumer exists yet. Numbered this Task 9, not Task 8: the FSD (gitignored, not tracked here before now) already used 'Task 8' for a planned Milestone 2 migration (guest_sessions/media, FSD change-note v2.9→v2.10) that has no corresponding code or tracker entry yet — a pre-existing drift between the FSD and this tracker, left as discovered rather than silently reconciled. docs/ is gitignored, so these edits are not versioned in git.</t>
+        </is>
+      </c>
+      <c r="G31" s="7" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H31" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="7" t="inlineStr">
+        <is>
+          <t>Milestone 8: RBAC foundation (cross-cutting platform work)</t>
+        </is>
+      </c>
+      <c r="B32" s="7" t="inlineStr">
         <is>
           <t>internal/db, services/rbac, services/event, cmd/api</t>
         </is>
       </c>
-      <c r="C28" s="7" t="inlineStr">
+      <c r="C32" s="7" t="inlineStr">
         <is>
           <t>T9.1</t>
         </is>
       </c>
-      <c r="D28" s="7" t="inlineStr">
+      <c r="D32" s="7" t="inlineStr">
         <is>
           <t>Implemented the RBAC foundation for real: migrations for roles/menus/dropdowns/actions/permissions, a services/rbac package (Postgres repository, Service resolving per-role menus/actions/dropdowns/preferences with a host-then-role-then-global fallback chain), GET /api/v1/auth/me and PATCH /api/v1/me/preferences, and events:create enforcement on the already-shipped POST /api/v1/events.</t>
         </is>
       </c>
-      <c r="E28" s="7" t="inlineStr">
+      <c r="E32" s="7" t="inlineStr">
         <is>
           <t>POST /api/v1/events now requires the events:create permission in addition to a host session; every existing host is granted it by default in the seed, so behavior is unchanged unless a permission is explicitly revoked.</t>
         </is>
       </c>
-      <c r="F28" s="7" t="inlineStr">
+      <c r="F32" s="7" t="inlineStr">
         <is>
           <t>Fallback-chain and ancestor-inclusion logic lives in Go (table-driven tested), not PL/pgSQL, matching this codebase's zero-stored-procedure convention; the one exception is a menu cycle-prevention trigger, a genuine data-integrity invariant a CHECK can't express. Seed data stays minimal and real: 2 flat menus (events_new, settings), 2 enforced permissions (events:create, profile:update); dropdowns and nested menus are schema-complete and tested but unseeded, since no real consumer exists yet. REST only, no gRPC, for /auth/me (fast-follow, mirrors Task 5's precedent). No permission-check caching (single API instance).</t>
         </is>
       </c>
-      <c r="G28" s="7" t="inlineStr">
+      <c r="G32" s="7" t="inlineStr">
         <is>
           <t>85ac425 cf5f3a8 e76992d b85cbb8 08d0812 1bc1ec4 68ae150 bb79173</t>
         </is>
       </c>
-      <c r="H28" s="7" t="inlineStr">
+      <c r="H32" s="7" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H28"/>
+  <autoFilter ref="A1:H32"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4540,11 +4912,19 @@
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F8" s="7" t="inlineStr"/>
-      <c r="G8" s="7" t="inlineStr"/>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>T8.2</t>
+        </is>
+      </c>
+      <c r="G8" s="7" t="inlineStr">
+        <is>
+          <t>guest sessions are only created for active, unexpired events (backend); the PWA camera page is not built yet</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
@@ -4569,17 +4949,17 @@
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>T8.1</t>
+          <t>T8.1, T8.2</t>
         </is>
       </c>
       <c r="G9" s="7" t="inlineStr">
         <is>
-          <t>guest_sessions table (one row per device session, optional nickname, no fingerprint); session creation and the guest cookie are not built yet</t>
+          <t>POST /api/v1/events/{event_id}/guest-session creates or resumes one anonymous session per browser via the sela_guest cookie; Redis stores only the token hash</t>
         </is>
       </c>
     </row>
@@ -4722,11 +5102,19 @@
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F14" s="7" t="inlineStr"/>
-      <c r="G14" s="7" t="inlineStr"/>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>T8.2</t>
+        </is>
+      </c>
+      <c r="G14" s="7" t="inlineStr">
+        <is>
+          <t>per-session quota enforced atomically in Redis at upload-URL issue and returned on failure; PWA shutter disabling not built</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
@@ -4838,11 +5226,19 @@
       </c>
       <c r="E18" s="7" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F18" s="7" t="inlineStr"/>
-      <c r="G18" s="7" t="inlineStr"/>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="F18" s="7" t="inlineStr">
+        <is>
+          <t>T8.1, T8.3</t>
+        </is>
+      </c>
+      <c r="G18" s="7" t="inlineStr">
+        <is>
+          <t>20 MB limit and format validation; JPEG/PNG/WebP only for now (HEIC, MP4, MOV refused until T8.4); multi-file UI not built</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
@@ -5012,11 +5408,19 @@
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F24" s="7" t="inlineStr"/>
-      <c r="G24" s="7" t="inlineStr"/>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="F24" s="7" t="inlineStr">
+        <is>
+          <t>T8.3</t>
+        </is>
+      </c>
+      <c r="G24" s="7" t="inlineStr">
+        <is>
+          <t>guest gallery query filters event_id + session_id in SQL (GET .../my-media); gallery UI is M3</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
@@ -5041,11 +5445,19 @@
       </c>
       <c r="E25" s="7" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F25" s="7" t="inlineStr"/>
-      <c r="G25" s="7" t="inlineStr"/>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="F25" s="7" t="inlineStr">
+        <is>
+          <t>T8.3</t>
+        </is>
+      </c>
+      <c r="G25" s="7" t="inlineStr">
+        <is>
+          <t>host gallery query checks ownership in SQL, no reveal gating (GET .../media); gallery UI is M3</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
@@ -5782,11 +6194,19 @@
       </c>
       <c r="E50" s="7" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F50" s="7" t="inlineStr"/>
-      <c r="G50" s="7" t="inlineStr"/>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="F50" s="7" t="inlineStr">
+        <is>
+          <t>T8.3</t>
+        </is>
+      </c>
+      <c r="G50" s="7" t="inlineStr">
+        <is>
+          <t>media only via short-lived pre-signed PUT/GET on a private bucket; separate media domain not done</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
@@ -5811,11 +6231,19 @@
       </c>
       <c r="E51" s="7" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F51" s="7" t="inlineStr"/>
-      <c r="G51" s="7" t="inlineStr"/>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="F51" s="7" t="inlineStr">
+        <is>
+          <t>T8.3</t>
+        </is>
+      </c>
+      <c r="G51" s="7" t="inlineStr">
+        <is>
+          <t>EXIF/GPS and all other metadata stripped from JPEG/PNG/WebP before storage; HEIC and video refused until T8.4</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
@@ -5840,11 +6268,19 @@
       </c>
       <c r="E52" s="7" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F52" s="7" t="inlineStr"/>
-      <c r="G52" s="7" t="inlineStr"/>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="F52" s="7" t="inlineStr">
+        <is>
+          <t>T8.3</t>
+        </is>
+      </c>
+      <c r="G52" s="7" t="inlineStr">
+        <is>
+          <t>magic bytes must match the declared type for JPEG/PNG/WebP</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
@@ -6063,11 +6499,19 @@
       </c>
       <c r="E59" s="7" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F59" s="7" t="inlineStr"/>
-      <c r="G59" s="7" t="inlineStr"/>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="F59" s="7" t="inlineStr">
+        <is>
+          <t>T8.3</t>
+        </is>
+      </c>
+      <c r="G59" s="7" t="inlineStr">
+        <is>
+          <t>X-Robots-Tag noindex, nofollow on every guest API route and the host gallery; web gallery pages not built</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:G59"/>

</xml_diff>

<commit_message>
docs: record Task 8.5 (guest rate limits) in the progress tracker
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/tracking/SELA_Progress_Tracker.xlsx
+++ b/docs/tracking/SELA_Progress_Tracker.xlsx
@@ -15,7 +15,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Tracker'!$A$1:$K$42</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Change Log'!$A$1:$H$32</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Change Log'!$A$1:$H$33</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Traceability'!$A$1:$G$59</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -516,7 +516,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Data as of 2026-09-23. Generated from docs/tracking/tracker.json and docs/FSD_Sela.md; do not edit this workbook by hand.</t>
+          <t>Data as of 2026-09-25. Generated from docs/tracking/tracker.json and docs/FSD_Sela.md; do not edit this workbook by hand.</t>
         </is>
       </c>
     </row>
@@ -578,7 +578,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Sheets: Summary (live counts), Tracker (one row per task and module), Change Log, Traceability (FR IDs).</t>
+          <t>Sheets: Summary (counts computed at build time), Tracker (one row per task and module), Change Log, Traceability (FR IDs).</t>
         </is>
       </c>
     </row>
@@ -648,29 +648,23 @@
           <t>Milestone 1: Host creates an event</t>
         </is>
       </c>
-      <c r="B2">
-        <f>COUNTIFS(Tracker!$A:$A,$A2,Tracker!$E:$E,B$1)</f>
-        <v/>
-      </c>
-      <c r="C2">
-        <f>COUNTIFS(Tracker!$A:$A,$A2,Tracker!$E:$E,C$1)</f>
-        <v/>
-      </c>
-      <c r="D2">
-        <f>COUNTIFS(Tracker!$A:$A,$A2,Tracker!$E:$E,D$1)</f>
-        <v/>
-      </c>
-      <c r="E2">
-        <f>COUNTIFS(Tracker!$A:$A,$A2,Tracker!$E:$E,E$1)</f>
-        <v/>
-      </c>
-      <c r="F2">
-        <f>SUM(B2:E2)</f>
-        <v/>
-      </c>
-      <c r="G2" s="5">
-        <f>IF(F2=0,0,E2/F2)</f>
-        <v/>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" t="n">
+        <v>22</v>
+      </c>
+      <c r="F2" t="n">
+        <v>24</v>
+      </c>
+      <c r="G2" s="5" t="n">
+        <v>0.9166666666666666</v>
       </c>
     </row>
     <row r="3">
@@ -679,29 +673,23 @@
           <t>Milestone 2: Guest captures and uploads</t>
         </is>
       </c>
-      <c r="B3">
-        <f>COUNTIFS(Tracker!$A:$A,$A3,Tracker!$E:$E,B$1)</f>
-        <v/>
-      </c>
-      <c r="C3">
-        <f>COUNTIFS(Tracker!$A:$A,$A3,Tracker!$E:$E,C$1)</f>
-        <v/>
-      </c>
-      <c r="D3">
-        <f>COUNTIFS(Tracker!$A:$A,$A3,Tracker!$E:$E,D$1)</f>
-        <v/>
-      </c>
-      <c r="E3">
-        <f>COUNTIFS(Tracker!$A:$A,$A3,Tracker!$E:$E,E$1)</f>
-        <v/>
-      </c>
-      <c r="F3">
-        <f>SUM(B3:E3)</f>
-        <v/>
-      </c>
-      <c r="G3" s="5">
-        <f>IF(F3=0,0,E3/F3)</f>
-        <v/>
+      <c r="B3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="n">
+        <v>4</v>
+      </c>
+      <c r="F3" t="n">
+        <v>6</v>
+      </c>
+      <c r="G3" s="5" t="n">
+        <v>0.6666666666666666</v>
       </c>
     </row>
     <row r="4">
@@ -710,29 +698,23 @@
           <t>Milestone 3: Role-correct gallery</t>
         </is>
       </c>
-      <c r="B4">
-        <f>COUNTIFS(Tracker!$A:$A,$A4,Tracker!$E:$E,B$1)</f>
-        <v/>
-      </c>
-      <c r="C4">
-        <f>COUNTIFS(Tracker!$A:$A,$A4,Tracker!$E:$E,C$1)</f>
-        <v/>
-      </c>
-      <c r="D4">
-        <f>COUNTIFS(Tracker!$A:$A,$A4,Tracker!$E:$E,D$1)</f>
-        <v/>
-      </c>
-      <c r="E4">
-        <f>COUNTIFS(Tracker!$A:$A,$A4,Tracker!$E:$E,E$1)</f>
-        <v/>
-      </c>
-      <c r="F4">
-        <f>SUM(B4:E4)</f>
-        <v/>
-      </c>
-      <c r="G4" s="5">
-        <f>IF(F4=0,0,E4/F4)</f>
-        <v/>
+      <c r="B4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G4" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -741,29 +723,23 @@
           <t>Milestone 4: Moderate and export</t>
         </is>
       </c>
-      <c r="B5">
-        <f>COUNTIFS(Tracker!$A:$A,$A5,Tracker!$E:$E,B$1)</f>
-        <v/>
-      </c>
-      <c r="C5">
-        <f>COUNTIFS(Tracker!$A:$A,$A5,Tracker!$E:$E,C$1)</f>
-        <v/>
-      </c>
-      <c r="D5">
-        <f>COUNTIFS(Tracker!$A:$A,$A5,Tracker!$E:$E,D$1)</f>
-        <v/>
-      </c>
-      <c r="E5">
-        <f>COUNTIFS(Tracker!$A:$A,$A5,Tracker!$E:$E,E$1)</f>
-        <v/>
-      </c>
-      <c r="F5">
-        <f>SUM(B5:E5)</f>
-        <v/>
-      </c>
-      <c r="G5" s="5">
-        <f>IF(F5=0,0,E5/F5)</f>
-        <v/>
+      <c r="B5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -772,29 +748,23 @@
           <t>Milestone 5: Plans and payment</t>
         </is>
       </c>
-      <c r="B6">
-        <f>COUNTIFS(Tracker!$A:$A,$A6,Tracker!$E:$E,B$1)</f>
-        <v/>
-      </c>
-      <c r="C6">
-        <f>COUNTIFS(Tracker!$A:$A,$A6,Tracker!$E:$E,C$1)</f>
-        <v/>
-      </c>
-      <c r="D6">
-        <f>COUNTIFS(Tracker!$A:$A,$A6,Tracker!$E:$E,D$1)</f>
-        <v/>
-      </c>
-      <c r="E6">
-        <f>COUNTIFS(Tracker!$A:$A,$A6,Tracker!$E:$E,E$1)</f>
-        <v/>
-      </c>
-      <c r="F6">
-        <f>SUM(B6:E6)</f>
-        <v/>
-      </c>
-      <c r="G6" s="5">
-        <f>IF(F6=0,0,E6/F6)</f>
-        <v/>
+      <c r="B6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -803,29 +773,23 @@
           <t>Milestone 6: Privacy and compliance readiness</t>
         </is>
       </c>
-      <c r="B7">
-        <f>COUNTIFS(Tracker!$A:$A,$A7,Tracker!$E:$E,B$1)</f>
-        <v/>
-      </c>
-      <c r="C7">
-        <f>COUNTIFS(Tracker!$A:$A,$A7,Tracker!$E:$E,C$1)</f>
-        <v/>
-      </c>
-      <c r="D7">
-        <f>COUNTIFS(Tracker!$A:$A,$A7,Tracker!$E:$E,D$1)</f>
-        <v/>
-      </c>
-      <c r="E7">
-        <f>COUNTIFS(Tracker!$A:$A,$A7,Tracker!$E:$E,E$1)</f>
-        <v/>
-      </c>
-      <c r="F7">
-        <f>SUM(B7:E7)</f>
-        <v/>
-      </c>
-      <c r="G7" s="5">
-        <f>IF(F7=0,0,E7/F7)</f>
-        <v/>
+      <c r="B7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -834,29 +798,23 @@
           <t>Milestone 7: Closed beta</t>
         </is>
       </c>
-      <c r="B8">
-        <f>COUNTIFS(Tracker!$A:$A,$A8,Tracker!$E:$E,B$1)</f>
-        <v/>
-      </c>
-      <c r="C8">
-        <f>COUNTIFS(Tracker!$A:$A,$A8,Tracker!$E:$E,C$1)</f>
-        <v/>
-      </c>
-      <c r="D8">
-        <f>COUNTIFS(Tracker!$A:$A,$A8,Tracker!$E:$E,D$1)</f>
-        <v/>
-      </c>
-      <c r="E8">
-        <f>COUNTIFS(Tracker!$A:$A,$A8,Tracker!$E:$E,E$1)</f>
-        <v/>
-      </c>
-      <c r="F8">
-        <f>SUM(B8:E8)</f>
-        <v/>
-      </c>
-      <c r="G8" s="5">
-        <f>IF(F8=0,0,E8/F8)</f>
-        <v/>
+      <c r="B8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -865,29 +823,23 @@
           <t>Milestone 8: RBAC foundation (cross-cutting platform work)</t>
         </is>
       </c>
-      <c r="B9">
-        <f>COUNTIFS(Tracker!$A:$A,$A9,Tracker!$E:$E,B$1)</f>
-        <v/>
-      </c>
-      <c r="C9">
-        <f>COUNTIFS(Tracker!$A:$A,$A9,Tracker!$E:$E,C$1)</f>
-        <v/>
-      </c>
-      <c r="D9">
-        <f>COUNTIFS(Tracker!$A:$A,$A9,Tracker!$E:$E,D$1)</f>
-        <v/>
-      </c>
-      <c r="E9">
-        <f>COUNTIFS(Tracker!$A:$A,$A9,Tracker!$E:$E,E$1)</f>
-        <v/>
-      </c>
-      <c r="F9">
-        <f>SUM(B9:E9)</f>
-        <v/>
-      </c>
-      <c r="G9" s="5">
-        <f>IF(F9=0,0,E9/F9)</f>
-        <v/>
+      <c r="B9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="n">
+        <v>3</v>
+      </c>
+      <c r="F9" t="n">
+        <v>3</v>
+      </c>
+      <c r="G9" s="5" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -896,29 +848,23 @@
           <t>Backlog: Should-have and later phases</t>
         </is>
       </c>
-      <c r="B10">
-        <f>COUNTIFS(Tracker!$A:$A,$A10,Tracker!$E:$E,B$1)</f>
-        <v/>
-      </c>
-      <c r="C10">
-        <f>COUNTIFS(Tracker!$A:$A,$A10,Tracker!$E:$E,C$1)</f>
-        <v/>
-      </c>
-      <c r="D10">
-        <f>COUNTIFS(Tracker!$A:$A,$A10,Tracker!$E:$E,D$1)</f>
-        <v/>
-      </c>
-      <c r="E10">
-        <f>COUNTIFS(Tracker!$A:$A,$A10,Tracker!$E:$E,E$1)</f>
-        <v/>
-      </c>
-      <c r="F10">
-        <f>SUM(B10:E10)</f>
-        <v/>
-      </c>
-      <c r="G10" s="5">
-        <f>IF(F10=0,0,E10/F10)</f>
-        <v/>
+      <c r="B10" t="n">
+        <v>3</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" t="n">
+        <v>3</v>
+      </c>
+      <c r="G10" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -927,29 +873,23 @@
           <t>All tasks</t>
         </is>
       </c>
-      <c r="B11">
-        <f>SUM(B2:B10)</f>
-        <v/>
-      </c>
-      <c r="C11">
-        <f>SUM(C2:C10)</f>
-        <v/>
-      </c>
-      <c r="D11">
-        <f>SUM(D2:D10)</f>
-        <v/>
-      </c>
-      <c r="E11">
-        <f>SUM(E2:E10)</f>
-        <v/>
-      </c>
-      <c r="F11">
-        <f>SUM(F2:F10)</f>
-        <v/>
-      </c>
-      <c r="G11" s="5">
-        <f>IF(F11=0,0,E11/F11)</f>
-        <v/>
+      <c r="B11" t="n">
+        <v>11</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" t="n">
+        <v>29</v>
+      </c>
+      <c r="F11" t="n">
+        <v>41</v>
+      </c>
+      <c r="G11" s="5" t="n">
+        <v>0.7073170731707317</v>
       </c>
     </row>
     <row r="13">
@@ -985,21 +925,17 @@
           <t>All FR IDs</t>
         </is>
       </c>
-      <c r="B14">
-        <f>COUNTIF(Traceability!$E:$E,B13)</f>
-        <v/>
-      </c>
-      <c r="C14">
-        <f>COUNTIF(Traceability!$E:$E,C13)</f>
-        <v/>
-      </c>
-      <c r="D14">
-        <f>COUNTIF(Traceability!$E:$E,D13)</f>
-        <v/>
-      </c>
-      <c r="E14">
-        <f>SUM(B14:D14)</f>
-        <v/>
+      <c r="B14" t="n">
+        <v>41</v>
+      </c>
+      <c r="C14" t="n">
+        <v>12</v>
+      </c>
+      <c r="D14" t="n">
+        <v>5</v>
+      </c>
+      <c r="E14" t="n">
+        <v>58</v>
       </c>
     </row>
   </sheetData>
@@ -2686,12 +2622,24 @@
       </c>
       <c r="E31" s="7" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F31" s="7" t="inlineStr"/>
-      <c r="G31" s="7" t="inlineStr"/>
-      <c r="H31" s="7" t="inlineStr"/>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F31" s="7" t="inlineStr">
+        <is>
+          <t>aba5d19 fc23d8c</t>
+        </is>
+      </c>
+      <c r="G31" s="7" t="inlineStr">
+        <is>
+          <t>bbd766d 420a2b4</t>
+        </is>
+      </c>
+      <c r="H31" s="7" t="inlineStr">
+        <is>
+          <t>85.2% (services/auth), 83.7% (services/media), 82.8% (cmd/api)</t>
+        </is>
+      </c>
       <c r="I31" s="7" t="inlineStr">
         <is>
           <t>FR-SEC.9</t>
@@ -2699,12 +2647,12 @@
       </c>
       <c r="J31" s="7" t="inlineStr">
         <is>
-          <t>Follow-up from T8.2/T8.3</t>
+          <t>auth.WindowLimiter (hashed rl:&lt;scope&gt;:&lt;sha256&gt; keys over CountWindow) + media.Limiter: 20 guest sessions/10 min/IP, 60 uploads/10 min/session, 300 uploads/10 min/IP; 429 + Retry-After; limiter errors fail closed (500). auth.ClientAddr exported (connection address only). scripts/check.sh passed (proto, gofmt, vet, lint, Go + web tests, e2e 10/10). Chore 47b0ad4 pins LF for *.go/*.sql.</t>
         </is>
       </c>
       <c r="K31" s="7" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
@@ -3257,7 +3205,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H32"/>
+  <dimension ref="A1:H33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -4454,74 +4402,74 @@
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>services/media, internal/config</t>
+          <t>services/auth, services/media</t>
         </is>
       </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>T8.2</t>
+          <t>T8.5</t>
         </is>
       </c>
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>Added anonymous guest sessions (POST /api/v1/events/{event_id}/guest-session, sela_guest cookie scoped to the event's API path) and an atomic Redis shot quota with rollback.</t>
+          <t>Added a reusable fixed-window limiter in auth and applied it to guest-session creation and upload requests (FR-SEC.9); FSD v2.14 (6, 8, 11.1).</t>
         </is>
       </c>
       <c r="E29" s="7" t="inlineStr">
         <is>
-          <t>New optional setting GUEST_SESSION_TTL (default 72h). New Redis keys guest:* and quota:*.</t>
+          <t>None. media.HTTPConfig gained an optional Limiter; nil disables limiting.</t>
         </is>
       </c>
       <c r="F29" s="7" t="inlineStr">
         <is>
-          <t>Session creation is a POST per FSD 6, not a side effect of GET /e/{short_code}, so link previews and crawlers create nothing. The cookie Path is /api/v1/events/{event_id} because a /e/ path would never reach the API. The quota counter reseeds from media rows, which stay the source of truth. Guest tokens reuse OTP_HMAC_KEY under their own domain prefix. The 72h TTL is a configurable default; the docs define none.</t>
+          <t>Limits are constants (not env) for now. Keys use the connection address only; behind a proxy all guests share a bucket unless the proxy preserves it. FR-SEC.9 stays Partial until share-link creation is limited.</t>
         </is>
       </c>
       <c r="G29" s="7" t="inlineStr">
         <is>
-          <t>83213fa 92f231d 69a73cb 4bb836c</t>
+          <t>aba5d19 bbd766d fc23d8c 420a2b4 47b0ad4</t>
         </is>
       </c>
       <c r="H29" s="7" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
         <is>
-          <t>Milestone 8: RBAC foundation (cross-cutting platform work)</t>
+          <t>Milestone 2: Guest captures and uploads</t>
         </is>
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>apps/web</t>
+          <t>services/media, internal/config</t>
         </is>
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>T9.2</t>
+          <t>T8.2</t>
         </is>
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>Added the rbac API client, a best-effort profile fetch in the root layout, a dynamic Nav component, a real dark theme palette, and a new /settings page with real EN/ID language and theme switching.</t>
+          <t>Added anonymous guest sessions (POST /api/v1/events/{event_id}/guest-session, sela_guest cookie scoped to the event's API path) and an atomic Redis shot quota with rollback.</t>
         </is>
       </c>
       <c r="E30" s="7" t="inlineStr">
         <is>
-          <t>The root layout's load() now returns a required profile field, which is merged into every page's PageData type (existing dashboard tests updated to pass profile: null).</t>
+          <t>New optional setting GUEST_SESSION_TTL (default 72h). New Redis keys guest:* and quota:*.</t>
         </is>
       </c>
       <c r="F30" s="7" t="inlineStr">
         <is>
-          <t>Only the nav and the new settings page get real i18n; the three existing host pages keep hardcoded Indonesian text (a larger, separate retrofit). A failed/401 profile fetch resolves to profile: null rather than throwing, so /auth/login never breaks. PATCH only sets concrete theme/language values, not 'clear back to inherited' (fast-follow).</t>
+          <t>Session creation is a POST per FSD 6, not a side effect of GET /e/{short_code}, so link previews and crawlers create nothing. The cookie Path is /api/v1/events/{event_id} because a /e/ path would never reach the API. The quota counter reseeds from media rows, which stay the source of truth. Guest tokens reuse OTP_HMAC_KEY under their own domain prefix. The 72h TTL is a configurable default; the docs define none.</t>
         </is>
       </c>
       <c r="G30" s="7" t="inlineStr">
         <is>
-          <t>14bc5fe e1cb469 6dea65a 23963e0 d98a473 694ba26 4be3c95 99c2c86 21fbdb5</t>
+          <t>83213fa 92f231d 69a73cb 4bb836c</t>
         </is>
       </c>
       <c r="H30" s="7" t="inlineStr">
@@ -4538,32 +4486,32 @@
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>docs, docs/tracking</t>
+          <t>apps/web</t>
         </is>
       </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
-          <t>T9.3</t>
+          <t>T9.2</t>
         </is>
       </c>
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>Verified the RBAC foundation against the real stack (Docker Redis+Mailpit, local Postgres, scripts/check.sh) and synced the FSD, CLAUDE.md and this tracker for Task 9.</t>
+          <t>Added the rbac API client, a best-effort profile fetch in the root layout, a dynamic Nav component, a real dark theme palette, and a new /settings page with real EN/ID language and theme switching.</t>
         </is>
       </c>
       <c r="E31" s="7" t="inlineStr">
         <is>
-          <t>None.</t>
+          <t>The root layout's load() now returns a required profile field, which is merged into every page's PageData type (existing dashboard tests updated to pass profile: null).</t>
         </is>
       </c>
       <c r="F31" s="7" t="inlineStr">
         <is>
-          <t>RBAC isn't tied to a numbered FR yet; no ID was invented (see FSD 11.1). Menu nesting and the dropdown tables are built and tested but unseeded, since no second real menu destination or dropdown consumer exists yet. Numbered this Task 9, not Task 8: the FSD (gitignored, not tracked here before now) already used 'Task 8' for a planned Milestone 2 migration (guest_sessions/media, FSD change-note v2.9→v2.10) that has no corresponding code or tracker entry yet — a pre-existing drift between the FSD and this tracker, left as discovered rather than silently reconciled. docs/ is gitignored, so these edits are not versioned in git.</t>
+          <t>Only the nav and the new settings page get real i18n; the three existing host pages keep hardcoded Indonesian text (a larger, separate retrofit). A failed/401 profile fetch resolves to profile: null rather than throwing, so /auth/login never breaks. PATCH only sets concrete theme/language values, not 'clear back to inherited' (fast-follow).</t>
         </is>
       </c>
       <c r="G31" s="7" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>14bc5fe e1cb469 6dea65a 23963e0 d98a473 694ba26 4be3c95 99c2c86 21fbdb5</t>
         </is>
       </c>
       <c r="H31" s="7" t="inlineStr">
@@ -4580,42 +4528,84 @@
       </c>
       <c r="B32" s="7" t="inlineStr">
         <is>
+          <t>docs, docs/tracking</t>
+        </is>
+      </c>
+      <c r="C32" s="7" t="inlineStr">
+        <is>
+          <t>T9.3</t>
+        </is>
+      </c>
+      <c r="D32" s="7" t="inlineStr">
+        <is>
+          <t>Verified the RBAC foundation against the real stack (Docker Redis+Mailpit, local Postgres, scripts/check.sh) and synced the FSD, CLAUDE.md and this tracker for Task 9.</t>
+        </is>
+      </c>
+      <c r="E32" s="7" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+      <c r="F32" s="7" t="inlineStr">
+        <is>
+          <t>RBAC isn't tied to a numbered FR yet; no ID was invented (see FSD 11.1). Menu nesting and the dropdown tables are built and tested but unseeded, since no second real menu destination or dropdown consumer exists yet. Numbered this Task 9, not Task 8: the FSD (gitignored, not tracked here before now) already used 'Task 8' for a planned Milestone 2 migration (guest_sessions/media, FSD change-note v2.9→v2.10) that has no corresponding code or tracker entry yet — a pre-existing drift between the FSD and this tracker, left as discovered rather than silently reconciled. docs/ is gitignored, so these edits are not versioned in git.</t>
+        </is>
+      </c>
+      <c r="G32" s="7" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H32" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>Milestone 8: RBAC foundation (cross-cutting platform work)</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
           <t>internal/db, services/rbac, services/event, cmd/api</t>
         </is>
       </c>
-      <c r="C32" s="7" t="inlineStr">
+      <c r="C33" s="7" t="inlineStr">
         <is>
           <t>T9.1</t>
         </is>
       </c>
-      <c r="D32" s="7" t="inlineStr">
+      <c r="D33" s="7" t="inlineStr">
         <is>
           <t>Implemented the RBAC foundation for real: migrations for roles/menus/dropdowns/actions/permissions, a services/rbac package (Postgres repository, Service resolving per-role menus/actions/dropdowns/preferences with a host-then-role-then-global fallback chain), GET /api/v1/auth/me and PATCH /api/v1/me/preferences, and events:create enforcement on the already-shipped POST /api/v1/events.</t>
         </is>
       </c>
-      <c r="E32" s="7" t="inlineStr">
+      <c r="E33" s="7" t="inlineStr">
         <is>
           <t>POST /api/v1/events now requires the events:create permission in addition to a host session; every existing host is granted it by default in the seed, so behavior is unchanged unless a permission is explicitly revoked.</t>
         </is>
       </c>
-      <c r="F32" s="7" t="inlineStr">
+      <c r="F33" s="7" t="inlineStr">
         <is>
           <t>Fallback-chain and ancestor-inclusion logic lives in Go (table-driven tested), not PL/pgSQL, matching this codebase's zero-stored-procedure convention; the one exception is a menu cycle-prevention trigger, a genuine data-integrity invariant a CHECK can't express. Seed data stays minimal and real: 2 flat menus (events_new, settings), 2 enforced permissions (events:create, profile:update); dropdowns and nested menus are schema-complete and tested but unseeded, since no real consumer exists yet. REST only, no gRPC, for /auth/me (fast-follow, mirrors Task 5's precedent). No permission-check caching (single API instance).</t>
         </is>
       </c>
-      <c r="G32" s="7" t="inlineStr">
+      <c r="G33" s="7" t="inlineStr">
         <is>
           <t>85ac425 cf5f3a8 e76992d b85cbb8 08d0812 1bc1ec4 68ae150 bb79173</t>
         </is>
       </c>
-      <c r="H32" s="7" t="inlineStr">
+      <c r="H33" s="7" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H32"/>
+  <autoFilter ref="A1:H33"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6467,12 +6457,12 @@
       </c>
       <c r="F58" s="7" t="inlineStr">
         <is>
-          <t>T3.5, T3.6</t>
+          <t>T3.5, T3.6, T8.5</t>
         </is>
       </c>
       <c r="G58" s="7" t="inlineStr">
         <is>
-          <t>Redis rate limiting on OTP endpoints; upload and share-link limits pending</t>
+          <t>Redis rate limiting on OTP endpoints and on guest-session creation and uploads (20 sessions/10 min/IP, 60 uploads/10 min/session, 300 uploads/10 min/IP, fail-closed); share-link creation limit pending</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: record Task 8.6 (guest short-code routes) in the progress tracker
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/tracking/SELA_Progress_Tracker.xlsx
+++ b/docs/tracking/SELA_Progress_Tracker.xlsx
@@ -14,8 +14,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Tracker'!$A$1:$K$42</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Change Log'!$A$1:$H$33</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Tracker'!$A$1:$K$43</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Change Log'!$A$1:$H$34</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Traceability'!$A$1:$G$59</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -683,13 +683,13 @@
         <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F3" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G3" s="5" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.7142857142857143</v>
       </c>
     </row>
     <row r="4">
@@ -883,13 +883,13 @@
         <v>1</v>
       </c>
       <c r="E11" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F11" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>0.7073170731707317</v>
+        <v>0.7142857142857143</v>
       </c>
     </row>
     <row r="13">
@@ -949,7 +949,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K42"/>
+  <dimension ref="A1:K43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2659,67 +2659,79 @@
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
         <is>
-          <t>Milestone 3: Role-correct gallery</t>
+          <t>Milestone 2: Guest captures and uploads</t>
         </is>
       </c>
       <c r="B32" s="7" t="inlineStr">
         <is>
-          <t>M3.1</t>
+          <t>T8.6</t>
         </is>
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>Milestone 3 (not yet planned) — Role-correct gallery, reveal timer, real-time channels</t>
+          <t>Guest short-code routes (pre-PWA) — Move the short-link resolver to /api/v1/e/{short_code} so the web app can own /e/{code} for the guest PWA page, and open a guest session straight from a short code</t>
         </is>
       </c>
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>services/gallery, services/realtime</t>
+          <t>services/event, services/media, cmd/api, apps/web (e2e)</t>
         </is>
       </c>
       <c r="E32" s="7" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F32" s="7" t="inlineStr"/>
-      <c r="G32" s="7" t="inlineStr"/>
-      <c r="H32" s="7" t="inlineStr"/>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F32" s="7" t="inlineStr">
+        <is>
+          <t>4651987 e7d5d53</t>
+        </is>
+      </c>
+      <c r="G32" s="7" t="inlineStr">
+        <is>
+          <t>b6509df 5a80691</t>
+        </is>
+      </c>
+      <c r="H32" s="7" t="inlineStr">
+        <is>
+          <t>91.3% (services/event), 84.4% (services/media), 82.8% (cmd/api)</t>
+        </is>
+      </c>
       <c r="I32" s="7" t="inlineStr">
         <is>
-          <t>FR-05.1-05.6</t>
+          <t>FR-01.3 FR-02.1 FR-02.2 FR-SEC.9</t>
         </is>
       </c>
       <c r="J32" s="7" t="inlineStr">
         <is>
-          <t>Host sees all media, guest only their own, WebSocket channels split by role</t>
+          <t>GET /api/v1/e/{short_code} replaces GET /e/{short_code} (handler, PublicEvent projection and identical 404s unchanged); the API no longer serves /e/. New POST /api/v1/e/{short_code}/guest-session with media.StartSessionByCode + Repository.GuestEventByShortCode (same SQL liveness filter over the unique short_code index) and media's own base62 screen, so media still never imports services/event. Shared joinEvent (service) and openSession (adapter) keep the two entry points from drifting. Cookie stays scoped to the resolved event id, so uploads receive it and resume goes through the {event_id} route. New route shares the guest-session rate-limit bucket, giving short-code probing a limit for the first time. Short link and QR still read {base}/e/{code}. Verified against a live API: resolver 200, retired /e/ 404, session 201 with Path=/api/v1/events/{resolved id}, unknown code 404; scripts/check.sh passed in full (proto drift, gofmt, vet, golangci-lint, Go tests, svelte-check 411 files 0 errors, web 184 tests, real-stack e2e 10/10).</t>
         </is>
       </c>
       <c r="K32" s="7" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
         <is>
-          <t>Milestone 4: Moderate and export</t>
+          <t>Milestone 3: Role-correct gallery</t>
         </is>
       </c>
       <c r="B33" s="7" t="inlineStr">
         <is>
-          <t>M4.1</t>
+          <t>M3.1</t>
         </is>
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>Milestone 4 (not yet planned) — Moderation and full-gallery ZIP export</t>
+          <t>Milestone 3 (not yet planned) — Role-correct gallery, reveal timer, real-time channels</t>
         </is>
       </c>
       <c r="D33" s="7" t="inlineStr">
         <is>
-          <t>services/gallery, services/media</t>
+          <t>services/gallery, services/realtime</t>
         </is>
       </c>
       <c r="E33" s="7" t="inlineStr">
@@ -2732,12 +2744,12 @@
       <c r="H33" s="7" t="inlineStr"/>
       <c r="I33" s="7" t="inlineStr">
         <is>
-          <t>FR-06.1-06.4, FR-07.1-07.3</t>
+          <t>FR-05.1-05.6</t>
         </is>
       </c>
       <c r="J33" s="7" t="inlineStr">
         <is>
-          <t>Hide/delete, asynchronous ZIP export, share links</t>
+          <t>Host sees all media, guest only their own, WebSocket channels split by role</t>
         </is>
       </c>
       <c r="K33" s="7" t="inlineStr">
@@ -2749,22 +2761,22 @@
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
         <is>
-          <t>Milestone 5: Plans and payment</t>
+          <t>Milestone 4: Moderate and export</t>
         </is>
       </c>
       <c r="B34" s="7" t="inlineStr">
         <is>
-          <t>M5.1</t>
+          <t>M4.1</t>
         </is>
       </c>
       <c r="C34" s="7" t="inlineStr">
         <is>
-          <t>Milestone 5 (not yet planned) — Plans, package recommendation and payment (QRIS, e-wallet, card)</t>
+          <t>Milestone 4 (not yet planned) — Moderation and full-gallery ZIP export</t>
         </is>
       </c>
       <c r="D34" s="7" t="inlineStr">
         <is>
-          <t>services/payment, services/event</t>
+          <t>services/gallery, services/media</t>
         </is>
       </c>
       <c r="E34" s="7" t="inlineStr">
@@ -2777,12 +2789,12 @@
       <c r="H34" s="7" t="inlineStr"/>
       <c r="I34" s="7" t="inlineStr">
         <is>
-          <t>FR-01.5, FR-01.6, FR-09.2, FR-09.3</t>
+          <t>FR-06.1-06.4, FR-07.1-07.3</t>
         </is>
       </c>
       <c r="J34" s="7" t="inlineStr">
         <is>
-          <t>Free and paid tiers by event scale; micro-payments; transaction history</t>
+          <t>Hide/delete, asynchronous ZIP export, share links</t>
         </is>
       </c>
       <c r="K34" s="7" t="inlineStr">
@@ -2794,22 +2806,22 @@
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
         <is>
-          <t>Milestone 6: Privacy and compliance readiness</t>
+          <t>Milestone 5: Plans and payment</t>
         </is>
       </c>
       <c r="B35" s="7" t="inlineStr">
         <is>
-          <t>M6.1</t>
+          <t>M5.1</t>
         </is>
       </c>
       <c r="C35" s="7" t="inlineStr">
         <is>
-          <t>Milestone 6 (not yet planned) — Privacy and compliance readiness</t>
+          <t>Milestone 5 (not yet planned) — Plans, package recommendation and payment (QRIS, e-wallet, card)</t>
         </is>
       </c>
       <c r="D35" s="7" t="inlineStr">
         <is>
-          <t>cross-cutting</t>
+          <t>services/payment, services/event</t>
         </is>
       </c>
       <c r="E35" s="7" t="inlineStr">
@@ -2822,12 +2834,12 @@
       <c r="H35" s="7" t="inlineStr"/>
       <c r="I35" s="7" t="inlineStr">
         <is>
-          <t>FR-SEC.1, FR-SEC.5-SEC.8, FR-SEC.10</t>
+          <t>FR-01.5, FR-01.6, FR-09.2, FR-09.3</t>
         </is>
       </c>
       <c r="J35" s="7" t="inlineStr">
         <is>
-          <t>PII column encryption with a blind index, audit log, retention and deletion, child-event defaults, noindex headers</t>
+          <t>Free and paid tiers by event scale; micro-payments; transaction history</t>
         </is>
       </c>
       <c r="K35" s="7" t="inlineStr">
@@ -2839,22 +2851,22 @@
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
         <is>
-          <t>Milestone 7: Closed beta</t>
+          <t>Milestone 6: Privacy and compliance readiness</t>
         </is>
       </c>
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t>M7.1</t>
+          <t>M6.1</t>
         </is>
       </c>
       <c r="C36" s="7" t="inlineStr">
         <is>
-          <t>Milestone 7 (not yet planned) — Closed beta across wedding, graduation and birthday events</t>
+          <t>Milestone 6 (not yet planned) — Privacy and compliance readiness</t>
         </is>
       </c>
       <c r="D36" s="7" t="inlineStr">
         <is>
-          <t>operations</t>
+          <t>cross-cutting</t>
         </is>
       </c>
       <c r="E36" s="7" t="inlineStr">
@@ -2865,10 +2877,14 @@
       <c r="F36" s="7" t="inlineStr"/>
       <c r="G36" s="7" t="inlineStr"/>
       <c r="H36" s="7" t="inlineStr"/>
-      <c r="I36" s="7" t="inlineStr"/>
+      <c r="I36" s="7" t="inlineStr">
+        <is>
+          <t>FR-SEC.1, FR-SEC.5-SEC.8, FR-SEC.10</t>
+        </is>
+      </c>
       <c r="J36" s="7" t="inlineStr">
         <is>
-          <t>Validate the hypothesis and fill the TBD success metrics in the PRD</t>
+          <t>PII column encryption with a blind index, audit log, retention and deletion, child-event defaults, noindex headers</t>
         </is>
       </c>
       <c r="K36" s="7" t="inlineStr">
@@ -2880,53 +2896,41 @@
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
         <is>
-          <t>Milestone 8: RBAC foundation (cross-cutting platform work)</t>
+          <t>Milestone 7: Closed beta</t>
         </is>
       </c>
       <c r="B37" s="7" t="inlineStr">
         <is>
-          <t>T9.1</t>
+          <t>M7.1</t>
         </is>
       </c>
       <c r="C37" s="7" t="inlineStr">
         <is>
-          <t>Task 9: RBAC foundation — RBAC schema (roles, menus, dropdowns, actions/permissions) and the services/rbac backend package; events:create gated on the already-shipped create-event route</t>
+          <t>Milestone 7 (not yet planned) — Closed beta across wedding, graduation and birthday events</t>
         </is>
       </c>
       <c r="D37" s="7" t="inlineStr">
         <is>
-          <t>internal/db (0004, 0005), services/rbac, services/event, cmd/api</t>
+          <t>operations</t>
         </is>
       </c>
       <c r="E37" s="7" t="inlineStr">
         <is>
-          <t>Completed</t>
-        </is>
-      </c>
-      <c r="F37" s="7" t="inlineStr">
-        <is>
-          <t>85ac425 e76992d 08d0812 68ae150</t>
-        </is>
-      </c>
-      <c r="G37" s="7" t="inlineStr">
-        <is>
-          <t>cf5f3a8 b85cbb8 1bc1ec4 bb79173</t>
-        </is>
-      </c>
-      <c r="H37" s="7" t="inlineStr">
-        <is>
-          <t>services/rbac 81.9%; services/event 91.3%; cmd/api 83.3%</t>
-        </is>
-      </c>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F37" s="7" t="inlineStr"/>
+      <c r="G37" s="7" t="inlineStr"/>
+      <c r="H37" s="7" t="inlineStr"/>
       <c r="I37" s="7" t="inlineStr"/>
       <c r="J37" s="7" t="inlineStr">
         <is>
-          <t>migrations 0004_rbac_foundation.sql, 0005_hosts_role_and_preferences.sql; services/rbac (types/postgres/service/http) with GET /api/v1/auth/me and PATCH /api/v1/me/preferences; RequirePermission wired onto POST /api/v1/events (events:create); seed limited to 2 menus (events_new, settings) and 2 enforced permissions (events:create, profile:update), every existing host granted both so no current behavior changes</t>
+          <t>Validate the hypothesis and fill the TBD success metrics in the PRD</t>
         </is>
       </c>
       <c r="K37" s="7" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-19</t>
         </is>
       </c>
     </row>
@@ -2938,17 +2942,17 @@
       </c>
       <c r="B38" s="7" t="inlineStr">
         <is>
-          <t>T9.2</t>
+          <t>T9.1</t>
         </is>
       </c>
       <c r="C38" s="7" t="inlineStr">
         <is>
-          <t>Task 9: RBAC foundation — Frontend: rbac API client, best-effort profile fetch in the root layout, dynamic Nav, dark theme palette, and the new /settings page with real EN/ID switching</t>
+          <t>Task 9: RBAC foundation — RBAC schema (roles, menus, dropdowns, actions/permissions) and the services/rbac backend package; events:create gated on the already-shipped create-event route</t>
         </is>
       </c>
       <c r="D38" s="7" t="inlineStr">
         <is>
-          <t>apps/web</t>
+          <t>internal/db (0004, 0005), services/rbac, services/event, cmd/api</t>
         </is>
       </c>
       <c r="E38" s="7" t="inlineStr">
@@ -2958,23 +2962,23 @@
       </c>
       <c r="F38" s="7" t="inlineStr">
         <is>
-          <t>14bc5fe 6dea65a 4be3c95</t>
+          <t>85ac425 e76992d 08d0812 68ae150</t>
         </is>
       </c>
       <c r="G38" s="7" t="inlineStr">
         <is>
-          <t>21fbdb5 e1cb469 23963e0 d98a473 694ba26 99c2c86</t>
+          <t>cf5f3a8 b85cbb8 1bc1ec4 bb79173</t>
         </is>
       </c>
       <c r="H38" s="7" t="inlineStr">
         <is>
-          <t>184 tests pass; 97.16% statements / 89.65% branches / 97.6% functions / 99.75% lines; svelte-check 0 errors/0 warnings</t>
+          <t>services/rbac 81.9%; services/event 91.3%; cmd/api 83.3%</t>
         </is>
       </c>
       <c r="I38" s="7" t="inlineStr"/>
       <c r="J38" s="7" t="inlineStr">
         <is>
-          <t>src/lib/api/rbac.ts; src/lib/components/Nav.svelte; :root[data-theme='dark'] palette in tokens.css; +layout.ts best-effort getProfile() (swallows a 401 so /auth/login never breaks); +layout.svelte renders Nav and sets document.documentElement.dataset.theme; src/routes/settings/+page.svelte (role, theme toggle, language toggle, own local EN/ID string table); the three pre-existing host pages keep their hardcoded Indonesian text unchanged</t>
+          <t>migrations 0004_rbac_foundation.sql, 0005_hosts_role_and_preferences.sql; services/rbac (types/postgres/service/http) with GET /api/v1/auth/me and PATCH /api/v1/me/preferences; RequirePermission wired onto POST /api/v1/events (events:create); seed limited to 2 menus (events_new, settings) and 2 enforced permissions (events:create, profile:update), every existing host granted both so no current behavior changes</t>
         </is>
       </c>
       <c r="K38" s="7" t="inlineStr">
@@ -2991,17 +2995,17 @@
       </c>
       <c r="B39" s="7" t="inlineStr">
         <is>
-          <t>T9.3</t>
+          <t>T9.2</t>
         </is>
       </c>
       <c r="C39" s="7" t="inlineStr">
         <is>
-          <t>Task 9: RBAC foundation — Real-stack verification and docs/tracking sync for Task 8</t>
+          <t>Task 9: RBAC foundation — Frontend: rbac API client, best-effort profile fetch in the root layout, dynamic Nav, dark theme palette, and the new /settings page with real EN/ID switching</t>
         </is>
       </c>
       <c r="D39" s="7" t="inlineStr">
         <is>
-          <t>docs, docs/tracking, CLAUDE.md</t>
+          <t>apps/web</t>
         </is>
       </c>
       <c r="E39" s="7" t="inlineStr">
@@ -3011,23 +3015,23 @@
       </c>
       <c r="F39" s="7" t="inlineStr">
         <is>
-          <t>n/a (documentation)</t>
+          <t>14bc5fe 6dea65a 4be3c95</t>
         </is>
       </c>
       <c r="G39" s="7" t="inlineStr">
         <is>
-          <t>n/a (docs/ is gitignored, not committed)</t>
+          <t>21fbdb5 e1cb469 23963e0 d98a473 694ba26 99c2c86</t>
         </is>
       </c>
       <c r="H39" s="7" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>184 tests pass; 97.16% statements / 89.65% branches / 97.6% functions / 99.75% lines; svelte-check 0 errors/0 warnings</t>
         </is>
       </c>
       <c r="I39" s="7" t="inlineStr"/>
       <c r="J39" s="7" t="inlineStr">
         <is>
-          <t>scripts/check.sh run against Docker Redis+Mailpit and a local Postgres (proto-gen --check, gofmt/vet/lint, go test -cover, svelte-check, vitest coverage, real-stack Playwright e2e); FSD 3.5/5/6/8.6/10.1/11.1 updates; CLAUDE.md bullets for services/rbac and the two new frontend surfaces; this tracker</t>
+          <t>src/lib/api/rbac.ts; src/lib/components/Nav.svelte; :root[data-theme='dark'] palette in tokens.css; +layout.ts best-effort getProfile() (swallows a 401 so /auth/login never breaks); +layout.svelte renders Nav and sets document.documentElement.dataset.theme; src/routes/settings/+page.svelte (role, theme toggle, language toggle, own local EN/ID string table); the three pre-existing host pages keep their hardcoded Indonesian text unchanged</t>
         </is>
       </c>
       <c r="K39" s="7" t="inlineStr">
@@ -3039,45 +3043,53 @@
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
         <is>
-          <t>Backlog: Should-have and later phases</t>
+          <t>Milestone 8: RBAC foundation (cross-cutting platform work)</t>
         </is>
       </c>
       <c r="B40" s="7" t="inlineStr">
         <is>
-          <t>BL.1</t>
+          <t>T9.3</t>
         </is>
       </c>
       <c r="C40" s="7" t="inlineStr">
         <is>
-          <t>Backlog: Notifications — Scheduled and transactional email/WhatsApp notifications</t>
+          <t>Task 9: RBAC foundation — Real-stack verification and docs/tracking sync for Task 8</t>
         </is>
       </c>
       <c r="D40" s="7" t="inlineStr">
         <is>
-          <t>services/notification</t>
+          <t>docs, docs/tracking, CLAUDE.md</t>
         </is>
       </c>
       <c r="E40" s="7" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F40" s="7" t="inlineStr"/>
-      <c r="G40" s="7" t="inlineStr"/>
-      <c r="H40" s="7" t="inlineStr"/>
-      <c r="I40" s="7" t="inlineStr">
-        <is>
-          <t>FR-08.1-08.2</t>
-        </is>
-      </c>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F40" s="7" t="inlineStr">
+        <is>
+          <t>n/a (documentation)</t>
+        </is>
+      </c>
+      <c r="G40" s="7" t="inlineStr">
+        <is>
+          <t>n/a (docs/ is gitignored, not committed)</t>
+        </is>
+      </c>
+      <c r="H40" s="7" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I40" s="7" t="inlineStr"/>
       <c r="J40" s="7" t="inlineStr">
         <is>
-          <t>Event reminders, reveal notices, expiry warnings</t>
+          <t>scripts/check.sh run against Docker Redis+Mailpit and a local Postgres (proto-gen --check, gofmt/vet/lint, go test -cover, svelte-check, vitest coverage, real-stack Playwright e2e); FSD 3.5/5/6/8.6/10.1/11.1 updates; CLAUDE.md bullets for services/rbac and the two new frontend surfaces; this tracker</t>
         </is>
       </c>
       <c r="K40" s="7" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
@@ -3089,17 +3101,17 @@
       </c>
       <c r="B41" s="7" t="inlineStr">
         <is>
-          <t>BL.2</t>
+          <t>BL.1</t>
         </is>
       </c>
       <c r="C41" s="7" t="inlineStr">
         <is>
-          <t>Backlog: Hall of Fame — Host-curated highlights visible to guests</t>
+          <t>Backlog: Notifications — Scheduled and transactional email/WhatsApp notifications</t>
         </is>
       </c>
       <c r="D41" s="7" t="inlineStr">
         <is>
-          <t>services/gallery</t>
+          <t>services/notification</t>
         </is>
       </c>
       <c r="E41" s="7" t="inlineStr">
@@ -3112,12 +3124,12 @@
       <c r="H41" s="7" t="inlineStr"/>
       <c r="I41" s="7" t="inlineStr">
         <is>
-          <t>FR-11.1-11.5</t>
+          <t>FR-08.1-08.2</t>
         </is>
       </c>
       <c r="J41" s="7" t="inlineStr">
         <is>
-          <t>Curation, ordering and sharing of the best photos</t>
+          <t>Event reminders, reveal notices, expiry warnings</t>
         </is>
       </c>
       <c r="K41" s="7" t="inlineStr">
@@ -3134,17 +3146,17 @@
       </c>
       <c r="B42" s="7" t="inlineStr">
         <is>
-          <t>BL.3</t>
+          <t>BL.2</t>
         </is>
       </c>
       <c r="C42" s="7" t="inlineStr">
         <is>
-          <t>Backlog: Personal/Instant Mode (v1.1) — Capture without an event and send results to several recipients</t>
+          <t>Backlog: Hall of Fame — Host-curated highlights visible to guests</t>
         </is>
       </c>
       <c r="D42" s="7" t="inlineStr">
         <is>
-          <t>apps/web, services/media</t>
+          <t>services/gallery</t>
         </is>
       </c>
       <c r="E42" s="7" t="inlineStr">
@@ -3157,23 +3169,68 @@
       <c r="H42" s="7" t="inlineStr"/>
       <c r="I42" s="7" t="inlineStr">
         <is>
+          <t>FR-11.1-11.5</t>
+        </is>
+      </c>
+      <c r="J42" s="7" t="inlineStr">
+        <is>
+          <t>Curation, ordering and sharing of the best photos</t>
+        </is>
+      </c>
+      <c r="K42" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="7" t="inlineStr">
+        <is>
+          <t>Backlog: Should-have and later phases</t>
+        </is>
+      </c>
+      <c r="B43" s="7" t="inlineStr">
+        <is>
+          <t>BL.3</t>
+        </is>
+      </c>
+      <c r="C43" s="7" t="inlineStr">
+        <is>
+          <t>Backlog: Personal/Instant Mode (v1.1) — Capture without an event and send results to several recipients</t>
+        </is>
+      </c>
+      <c r="D43" s="7" t="inlineStr">
+        <is>
+          <t>apps/web, services/media</t>
+        </is>
+      </c>
+      <c r="E43" s="7" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F43" s="7" t="inlineStr"/>
+      <c r="G43" s="7" t="inlineStr"/>
+      <c r="H43" s="7" t="inlineStr"/>
+      <c r="I43" s="7" t="inlineStr">
+        <is>
           <t>FR-10.1-10.7</t>
         </is>
       </c>
-      <c r="J42" s="7" t="inlineStr">
+      <c r="J43" s="7" t="inlineStr">
         <is>
           <t>Deferred until Event Mode is stable</t>
         </is>
       </c>
-      <c r="K42" s="7" t="inlineStr">
+      <c r="K43" s="7" t="inlineStr">
         <is>
           <t>2026-09-19</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K42"/>
-  <conditionalFormatting sqref="E2:E42">
+  <autoFilter ref="A1:K43"/>
+  <conditionalFormatting sqref="E2:E43">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$E2="Not Started"</formula>
     </cfRule>
@@ -3191,7 +3248,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="E2:E42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E2:E43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Not Started,In Progress,Pending Verification,Completed"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3205,7 +3262,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H33"/>
+  <dimension ref="A1:H34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -4444,74 +4501,74 @@
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>services/media, internal/config</t>
+          <t>services/event, services/media, cmd/api, apps/web</t>
         </is>
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>T8.2</t>
+          <t>T8.6</t>
         </is>
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>Added anonymous guest sessions (POST /api/v1/events/{event_id}/guest-session, sela_guest cookie scoped to the event's API path) and an atomic Redis shot quota with rollback.</t>
+          <t>Moved the short-link resolver to GET /api/v1/e/{short_code} and added POST /api/v1/e/{short_code}/guest-session, so /e/{code} is free for the guest PWA page and a scanned QR opens a session in one round trip; FSD v2.15 (6, 8.6, 11.1).</t>
         </is>
       </c>
       <c r="E30" s="7" t="inlineStr">
         <is>
-          <t>New optional setting GUEST_SESSION_TTL (default 72h). New Redis keys guest:* and quota:*.</t>
+          <t>GET /e/{short_code} is no longer served by the API. Only two call sites used it (cmd/api/e2e_test.go, apps/web host e2e); both moved. The short link and QR are unchanged and still read {base}/e/{code}. media.Guests gained StartSessionByCode, so the three stub implementations were updated.</t>
         </is>
       </c>
       <c r="F30" s="7" t="inlineStr">
         <is>
-          <t>Session creation is a POST per FSD 6, not a side effect of GET /e/{short_code}, so link previews and crawlers create nothing. The cookie Path is /api/v1/events/{event_id} because a /e/ path would never reach the API. The quota counter reseeds from media rows, which stay the source of truth. Guest tokens reuse OTP_HMAC_KEY under their own domain prefix. The 72h TTL is a configurable default; the docs define none.</t>
+          <t>Neither route can nest under /api/v1/events/: ServeMux rejects a two-segment pattern there as conflicting with {id}/qr.png, and a by-code guest-session route would collide with {event_id}/media/{media_id}. /api/v1/e/ was chosen to mirror the guest-facing link. The by-code route cannot resume, because the guest cookie is scoped to /api/v1/events/{event_id} and is never sent to it; it is first-contact only and returns event_id so the client resumes through the {event_id} route. Widening the cookie path was rejected to keep the FSD 8.6 scope. media keeps its own base62 pattern rather than importing services/event.</t>
         </is>
       </c>
       <c r="G30" s="7" t="inlineStr">
         <is>
-          <t>83213fa 92f231d 69a73cb 4bb836c</t>
+          <t>4651987 b6509df e7d5d53 5a80691</t>
         </is>
       </c>
       <c r="H30" s="7" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
         <is>
-          <t>Milestone 8: RBAC foundation (cross-cutting platform work)</t>
+          <t>Milestone 2: Guest captures and uploads</t>
         </is>
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>apps/web</t>
+          <t>services/media, internal/config</t>
         </is>
       </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
-          <t>T9.2</t>
+          <t>T8.2</t>
         </is>
       </c>
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>Added the rbac API client, a best-effort profile fetch in the root layout, a dynamic Nav component, a real dark theme palette, and a new /settings page with real EN/ID language and theme switching.</t>
+          <t>Added anonymous guest sessions (POST /api/v1/events/{event_id}/guest-session, sela_guest cookie scoped to the event's API path) and an atomic Redis shot quota with rollback.</t>
         </is>
       </c>
       <c r="E31" s="7" t="inlineStr">
         <is>
-          <t>The root layout's load() now returns a required profile field, which is merged into every page's PageData type (existing dashboard tests updated to pass profile: null).</t>
+          <t>New optional setting GUEST_SESSION_TTL (default 72h). New Redis keys guest:* and quota:*.</t>
         </is>
       </c>
       <c r="F31" s="7" t="inlineStr">
         <is>
-          <t>Only the nav and the new settings page get real i18n; the three existing host pages keep hardcoded Indonesian text (a larger, separate retrofit). A failed/401 profile fetch resolves to profile: null rather than throwing, so /auth/login never breaks. PATCH only sets concrete theme/language values, not 'clear back to inherited' (fast-follow).</t>
+          <t>Session creation is a POST per FSD 6, not a side effect of GET /e/{short_code}, so link previews and crawlers create nothing. The cookie Path is /api/v1/events/{event_id} because a /e/ path would never reach the API. The quota counter reseeds from media rows, which stay the source of truth. Guest tokens reuse OTP_HMAC_KEY under their own domain prefix. The 72h TTL is a configurable default; the docs define none.</t>
         </is>
       </c>
       <c r="G31" s="7" t="inlineStr">
         <is>
-          <t>14bc5fe e1cb469 6dea65a 23963e0 d98a473 694ba26 4be3c95 99c2c86 21fbdb5</t>
+          <t>83213fa 92f231d 69a73cb 4bb836c</t>
         </is>
       </c>
       <c r="H31" s="7" t="inlineStr">
@@ -4528,32 +4585,32 @@
       </c>
       <c r="B32" s="7" t="inlineStr">
         <is>
-          <t>docs, docs/tracking</t>
+          <t>apps/web</t>
         </is>
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>T9.3</t>
+          <t>T9.2</t>
         </is>
       </c>
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>Verified the RBAC foundation against the real stack (Docker Redis+Mailpit, local Postgres, scripts/check.sh) and synced the FSD, CLAUDE.md and this tracker for Task 9.</t>
+          <t>Added the rbac API client, a best-effort profile fetch in the root layout, a dynamic Nav component, a real dark theme palette, and a new /settings page with real EN/ID language and theme switching.</t>
         </is>
       </c>
       <c r="E32" s="7" t="inlineStr">
         <is>
-          <t>None.</t>
+          <t>The root layout's load() now returns a required profile field, which is merged into every page's PageData type (existing dashboard tests updated to pass profile: null).</t>
         </is>
       </c>
       <c r="F32" s="7" t="inlineStr">
         <is>
-          <t>RBAC isn't tied to a numbered FR yet; no ID was invented (see FSD 11.1). Menu nesting and the dropdown tables are built and tested but unseeded, since no second real menu destination or dropdown consumer exists yet. Numbered this Task 9, not Task 8: the FSD (gitignored, not tracked here before now) already used 'Task 8' for a planned Milestone 2 migration (guest_sessions/media, FSD change-note v2.9→v2.10) that has no corresponding code or tracker entry yet — a pre-existing drift between the FSD and this tracker, left as discovered rather than silently reconciled. docs/ is gitignored, so these edits are not versioned in git.</t>
+          <t>Only the nav and the new settings page get real i18n; the three existing host pages keep hardcoded Indonesian text (a larger, separate retrofit). A failed/401 profile fetch resolves to profile: null rather than throwing, so /auth/login never breaks. PATCH only sets concrete theme/language values, not 'clear back to inherited' (fast-follow).</t>
         </is>
       </c>
       <c r="G32" s="7" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>14bc5fe e1cb469 6dea65a 23963e0 d98a473 694ba26 4be3c95 99c2c86 21fbdb5</t>
         </is>
       </c>
       <c r="H32" s="7" t="inlineStr">
@@ -4570,42 +4627,84 @@
       </c>
       <c r="B33" s="7" t="inlineStr">
         <is>
+          <t>docs, docs/tracking</t>
+        </is>
+      </c>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>T9.3</t>
+        </is>
+      </c>
+      <c r="D33" s="7" t="inlineStr">
+        <is>
+          <t>Verified the RBAC foundation against the real stack (Docker Redis+Mailpit, local Postgres, scripts/check.sh) and synced the FSD, CLAUDE.md and this tracker for Task 9.</t>
+        </is>
+      </c>
+      <c r="E33" s="7" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+      <c r="F33" s="7" t="inlineStr">
+        <is>
+          <t>RBAC isn't tied to a numbered FR yet; no ID was invented (see FSD 11.1). Menu nesting and the dropdown tables are built and tested but unseeded, since no second real menu destination or dropdown consumer exists yet. Numbered this Task 9, not Task 8: the FSD (gitignored, not tracked here before now) already used 'Task 8' for a planned Milestone 2 migration (guest_sessions/media, FSD change-note v2.9→v2.10) that has no corresponding code or tracker entry yet — a pre-existing drift between the FSD and this tracker, left as discovered rather than silently reconciled. docs/ is gitignored, so these edits are not versioned in git.</t>
+        </is>
+      </c>
+      <c r="G33" s="7" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H33" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="7" t="inlineStr">
+        <is>
+          <t>Milestone 8: RBAC foundation (cross-cutting platform work)</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="inlineStr">
+        <is>
           <t>internal/db, services/rbac, services/event, cmd/api</t>
         </is>
       </c>
-      <c r="C33" s="7" t="inlineStr">
+      <c r="C34" s="7" t="inlineStr">
         <is>
           <t>T9.1</t>
         </is>
       </c>
-      <c r="D33" s="7" t="inlineStr">
+      <c r="D34" s="7" t="inlineStr">
         <is>
           <t>Implemented the RBAC foundation for real: migrations for roles/menus/dropdowns/actions/permissions, a services/rbac package (Postgres repository, Service resolving per-role menus/actions/dropdowns/preferences with a host-then-role-then-global fallback chain), GET /api/v1/auth/me and PATCH /api/v1/me/preferences, and events:create enforcement on the already-shipped POST /api/v1/events.</t>
         </is>
       </c>
-      <c r="E33" s="7" t="inlineStr">
+      <c r="E34" s="7" t="inlineStr">
         <is>
           <t>POST /api/v1/events now requires the events:create permission in addition to a host session; every existing host is granted it by default in the seed, so behavior is unchanged unless a permission is explicitly revoked.</t>
         </is>
       </c>
-      <c r="F33" s="7" t="inlineStr">
+      <c r="F34" s="7" t="inlineStr">
         <is>
           <t>Fallback-chain and ancestor-inclusion logic lives in Go (table-driven tested), not PL/pgSQL, matching this codebase's zero-stored-procedure convention; the one exception is a menu cycle-prevention trigger, a genuine data-integrity invariant a CHECK can't express. Seed data stays minimal and real: 2 flat menus (events_new, settings), 2 enforced permissions (events:create, profile:update); dropdowns and nested menus are schema-complete and tested but unseeded, since no real consumer exists yet. REST only, no gRPC, for /auth/me (fast-follow, mirrors Task 5's precedent). No permission-check caching (single API instance).</t>
         </is>
       </c>
-      <c r="G33" s="7" t="inlineStr">
+      <c r="G34" s="7" t="inlineStr">
         <is>
           <t>85ac425 cf5f3a8 e76992d b85cbb8 08d0812 1bc1ec4 68ae150 bb79173</t>
         </is>
       </c>
-      <c r="H33" s="7" t="inlineStr">
+      <c r="H34" s="7" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H33"/>
+  <autoFilter ref="A1:H34"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>